<commit_message>
Update MVP 1.0 version planning baseline
</commit_message>
<xml_diff>
--- a/docs/MVP 0.9 项目管理/01_需求与版本规划/EOR MVP 1.0 目标版本规划 V1.1.xlsx
+++ b/docs/MVP 0.9 项目管理/01_需求与版本规划/EOR MVP 1.0 目标版本规划 V1.1.xlsx
@@ -18,7 +18,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">人物设定!$A$1:$C$19</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'MVP 1.0特性清单'!$A$3:$G$104</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'MVP 1.0特性清单'!$A$3:$G$105</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1162" uniqueCount="834">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1168" uniqueCount="837">
   <si>
     <t>人物属性</t>
   </si>
@@ -1334,6 +1334,12 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="宋体"/>
+        <charset val="134"/>
+      </rPr>
       <t>基于</t>
     </r>
     <r>
@@ -1378,6 +1384,44 @@
   </si>
   <si>
     <t>启动图形用户界面开发，先实现核心面板（主菜单、回合状态、地图视图）。</t>
+  </si>
+  <si>
+    <t>GUI-P0-02</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">P0 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="宋体"/>
+        <charset val="134"/>
+      </rPr>
+      <t>核心</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Segoe UI"/>
+        <charset val="134"/>
+      </rPr>
+      <t xml:space="preserve"> GUI </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="宋体"/>
+        <charset val="134"/>
+      </rPr>
+      <t>闭环</t>
+    </r>
+  </si>
+  <si>
+    <t>进入 P1 前，应该先补一个 “P0 核心 GUI 闭环”，让 MVP0.7/P0 主流程能在 GUI 上跑成功；但不要把所有 CLI 功能都完整迁移完再开发 P1。这样既降低 P1 GUI 返工，又不会被 GUI 产品化拖住主线。包含7个子任务；</t>
   </si>
   <si>
     <t>七、其他细节</t>
@@ -3635,13 +3679,13 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="9"/>
+      <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Consolas"/>
       <charset val="134"/>
     </font>
     <font>
-      <sz val="10"/>
+      <sz val="9"/>
       <color rgb="FF000000"/>
       <name val="Consolas"/>
       <charset val="134"/>
@@ -4241,7 +4285,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="49">
+  <cellXfs count="50">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -4346,6 +4390,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -4663,7 +4710,7 @@
     </dxf>
   </dxfs>
   <tableStyles count="2" defaultTableStyle="TableStylePreset3_Accent1 1" defaultPivotStyle="PivotStylePreset2_Accent1 1">
-    <tableStyle name="TableStylePreset3_Accent1 1" pivot="0" count="7" xr9:uid="{39ACA3F8-808E-4243-91E8-0A655D6BE38B}">
+    <tableStyle name="TableStylePreset3_Accent1 1" pivot="0" count="7" xr9:uid="{DCD53CD2-7D63-465F-8282-B831EBB5EED1}">
       <tableStyleElement type="wholeTable" dxfId="7"/>
       <tableStyleElement type="headerRow" dxfId="6"/>
       <tableStyleElement type="totalRow" dxfId="5"/>
@@ -4672,7 +4719,7 @@
       <tableStyleElement type="firstRowStripe" dxfId="2"/>
       <tableStyleElement type="firstColumnStripe" dxfId="1"/>
     </tableStyle>
-    <tableStyle name="PivotStylePreset2_Accent1 1" table="0" count="10" xr9:uid="{55A37C8B-DAE7-43DE-B459-7D738757185F}">
+    <tableStyle name="PivotStylePreset2_Accent1 1" table="0" count="10" xr9:uid="{D209FF72-8775-4799-A746-0B9339E74356}">
       <tableStyleElement type="headerRow" dxfId="17"/>
       <tableStyleElement type="totalRow" dxfId="16"/>
       <tableStyleElement type="firstRowStripe" dxfId="15"/>
@@ -4954,325 +5001,325 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5">
-      <c r="A1" s="44" t="s">
+      <c r="A1" s="45" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="44" t="s">
+      <c r="B1" s="45" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="44" t="s">
+      <c r="C1" s="45" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="44" t="s">
+      <c r="D1" s="45" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="44" t="s">
+      <c r="E1" s="45" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="2" spans="1:5">
-      <c r="A2" s="45" t="s">
+      <c r="A2" s="46" t="s">
         <v>5</v>
       </c>
-      <c r="B2" s="46" t="s">
+      <c r="B2" s="47" t="s">
         <v>6</v>
       </c>
-      <c r="C2" s="46" t="s">
+      <c r="C2" s="47" t="s">
         <v>7</v>
       </c>
-      <c r="D2" s="46" t="s">
+      <c r="D2" s="47" t="s">
         <v>8</v>
       </c>
-      <c r="E2" s="46" t="s">
+      <c r="E2" s="47" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="3" spans="1:5">
-      <c r="A3" s="45" t="s">
+      <c r="A3" s="46" t="s">
         <v>10</v>
       </c>
-      <c r="B3" s="46" t="s">
+      <c r="B3" s="47" t="s">
         <v>11</v>
       </c>
-      <c r="C3" s="46" t="s">
+      <c r="C3" s="47" t="s">
         <v>7</v>
       </c>
-      <c r="D3" s="46" t="s">
+      <c r="D3" s="47" t="s">
         <v>8</v>
       </c>
-      <c r="E3" s="46" t="s">
+      <c r="E3" s="47" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="4" spans="1:5">
-      <c r="A4" s="45" t="s">
+      <c r="A4" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="B4" s="46" t="s">
+      <c r="B4" s="47" t="s">
         <v>13</v>
       </c>
-      <c r="C4" s="46" t="s">
+      <c r="C4" s="47" t="s">
         <v>7</v>
       </c>
-      <c r="D4" s="46" t="s">
+      <c r="D4" s="47" t="s">
         <v>8</v>
       </c>
-      <c r="E4" s="46" t="s">
+      <c r="E4" s="47" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="5" spans="1:5">
-      <c r="A5" s="45" t="s">
+      <c r="A5" s="46" t="s">
         <v>14</v>
       </c>
-      <c r="B5" s="46" t="s">
+      <c r="B5" s="47" t="s">
         <v>15</v>
       </c>
-      <c r="C5" s="46" t="s">
+      <c r="C5" s="47" t="s">
         <v>7</v>
       </c>
-      <c r="D5" s="46" t="s">
+      <c r="D5" s="47" t="s">
         <v>8</v>
       </c>
-      <c r="E5" s="46" t="s">
+      <c r="E5" s="47" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="6" spans="1:5">
-      <c r="A6" s="47" t="s">
+      <c r="A6" s="48" t="s">
         <v>16</v>
       </c>
-      <c r="B6" s="46" t="s">
+      <c r="B6" s="47" t="s">
         <v>17</v>
       </c>
-      <c r="C6" s="46" t="s">
+      <c r="C6" s="47" t="s">
         <v>18</v>
       </c>
-      <c r="D6" s="46" t="s">
+      <c r="D6" s="47" t="s">
         <v>19</v>
       </c>
-      <c r="E6" s="46" t="s">
+      <c r="E6" s="47" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="7" spans="1:5">
-      <c r="A7" s="47" t="s">
+      <c r="A7" s="48" t="s">
         <v>21</v>
       </c>
-      <c r="B7" s="46" t="s">
+      <c r="B7" s="47" t="s">
         <v>22</v>
       </c>
-      <c r="C7" s="46" t="s">
+      <c r="C7" s="47" t="s">
         <v>18</v>
       </c>
-      <c r="D7" s="46" t="s">
+      <c r="D7" s="47" t="s">
         <v>23</v>
       </c>
-      <c r="E7" s="46" t="s">
+      <c r="E7" s="47" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="8" spans="1:5">
-      <c r="A8" s="47" t="s">
+      <c r="A8" s="48" t="s">
         <v>25</v>
       </c>
-      <c r="B8" s="46" t="s">
+      <c r="B8" s="47" t="s">
         <v>26</v>
       </c>
-      <c r="C8" s="46" t="s">
+      <c r="C8" s="47" t="s">
         <v>18</v>
       </c>
-      <c r="D8" s="46" t="s">
+      <c r="D8" s="47" t="s">
         <v>8</v>
       </c>
-      <c r="E8" s="46" t="s">
+      <c r="E8" s="47" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="9" spans="1:5">
-      <c r="A9" s="48" t="s">
+      <c r="A9" s="49" t="s">
         <v>28</v>
       </c>
-      <c r="B9" s="46" t="s">
+      <c r="B9" s="47" t="s">
         <v>29</v>
       </c>
-      <c r="C9" s="46" t="s">
+      <c r="C9" s="47" t="s">
         <v>18</v>
       </c>
-      <c r="D9" s="46" t="s">
+      <c r="D9" s="47" t="s">
         <v>23</v>
       </c>
-      <c r="E9" s="46" t="s">
+      <c r="E9" s="47" t="s">
         <v>30</v>
       </c>
     </row>
     <row r="10" spans="1:5">
-      <c r="A10" s="48" t="s">
+      <c r="A10" s="49" t="s">
         <v>31</v>
       </c>
-      <c r="B10" s="46" t="s">
+      <c r="B10" s="47" t="s">
         <v>32</v>
       </c>
-      <c r="C10" s="46" t="s">
+      <c r="C10" s="47" t="s">
         <v>33</v>
       </c>
-      <c r="D10" s="46" t="s">
+      <c r="D10" s="47" t="s">
         <v>23</v>
       </c>
-      <c r="E10" s="46" t="s">
+      <c r="E10" s="47" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="11" spans="1:5">
-      <c r="A11" s="48" t="s">
+      <c r="A11" s="49" t="s">
         <v>35</v>
       </c>
-      <c r="B11" s="46" t="s">
+      <c r="B11" s="47" t="s">
         <v>36</v>
       </c>
-      <c r="C11" s="46" t="s">
+      <c r="C11" s="47" t="s">
         <v>18</v>
       </c>
-      <c r="D11" s="46" t="s">
+      <c r="D11" s="47" t="s">
         <v>37</v>
       </c>
-      <c r="E11" s="46" t="s">
+      <c r="E11" s="47" t="s">
         <v>38</v>
       </c>
     </row>
     <row r="12" spans="1:5">
-      <c r="A12" s="48" t="s">
+      <c r="A12" s="49" t="s">
         <v>39</v>
       </c>
-      <c r="B12" s="46" t="s">
+      <c r="B12" s="47" t="s">
         <v>40</v>
       </c>
-      <c r="C12" s="46" t="s">
+      <c r="C12" s="47" t="s">
         <v>18</v>
       </c>
-      <c r="D12" s="46" t="s">
+      <c r="D12" s="47" t="s">
         <v>41</v>
       </c>
-      <c r="E12" s="46" t="s">
+      <c r="E12" s="47" t="s">
         <v>42</v>
       </c>
     </row>
     <row r="13" spans="1:5">
-      <c r="A13" s="48" t="s">
+      <c r="A13" s="49" t="s">
         <v>43</v>
       </c>
-      <c r="B13" s="46" t="s">
+      <c r="B13" s="47" t="s">
         <v>44</v>
       </c>
-      <c r="C13" s="46" t="s">
+      <c r="C13" s="47" t="s">
         <v>7</v>
       </c>
-      <c r="D13" s="46" t="s">
+      <c r="D13" s="47" t="s">
         <v>45</v>
       </c>
-      <c r="E13" s="46" t="s">
+      <c r="E13" s="47" t="s">
         <v>46</v>
       </c>
     </row>
     <row r="14" spans="1:5">
-      <c r="A14" s="48" t="s">
+      <c r="A14" s="49" t="s">
         <v>47</v>
       </c>
-      <c r="B14" s="46" t="s">
+      <c r="B14" s="47" t="s">
         <v>48</v>
       </c>
-      <c r="C14" s="46" t="s">
+      <c r="C14" s="47" t="s">
         <v>7</v>
       </c>
-      <c r="D14" s="46" t="s">
+      <c r="D14" s="47" t="s">
         <v>8</v>
       </c>
-      <c r="E14" s="46" t="s">
+      <c r="E14" s="47" t="s">
         <v>49</v>
       </c>
     </row>
     <row r="15" spans="1:5">
-      <c r="A15" s="48" t="s">
+      <c r="A15" s="49" t="s">
         <v>50</v>
       </c>
-      <c r="B15" s="46" t="s">
+      <c r="B15" s="47" t="s">
         <v>51</v>
       </c>
-      <c r="C15" s="46" t="s">
+      <c r="C15" s="47" t="s">
         <v>7</v>
       </c>
-      <c r="D15" s="46" t="s">
+      <c r="D15" s="47" t="s">
         <v>8</v>
       </c>
-      <c r="E15" s="46" t="s">
+      <c r="E15" s="47" t="s">
         <v>49</v>
       </c>
     </row>
     <row r="16" spans="1:5">
-      <c r="A16" s="48" t="s">
+      <c r="A16" s="49" t="s">
         <v>52</v>
       </c>
-      <c r="B16" s="46" t="s">
+      <c r="B16" s="47" t="s">
         <v>53</v>
       </c>
-      <c r="C16" s="46" t="s">
+      <c r="C16" s="47" t="s">
         <v>7</v>
       </c>
-      <c r="D16" s="46" t="s">
+      <c r="D16" s="47" t="s">
         <v>8</v>
       </c>
-      <c r="E16" s="46" t="s">
+      <c r="E16" s="47" t="s">
         <v>49</v>
       </c>
     </row>
     <row r="17" spans="1:5">
-      <c r="A17" s="48" t="s">
+      <c r="A17" s="49" t="s">
         <v>54</v>
       </c>
-      <c r="B17" s="46" t="s">
+      <c r="B17" s="47" t="s">
         <v>55</v>
       </c>
-      <c r="C17" s="46" t="s">
+      <c r="C17" s="47" t="s">
         <v>7</v>
       </c>
-      <c r="D17" s="46" t="s">
+      <c r="D17" s="47" t="s">
         <v>56</v>
       </c>
-      <c r="E17" s="46" t="s">
+      <c r="E17" s="47" t="s">
         <v>57</v>
       </c>
     </row>
     <row r="18" spans="1:5">
-      <c r="A18" s="48" t="s">
+      <c r="A18" s="49" t="s">
         <v>58</v>
       </c>
-      <c r="B18" s="46" t="s">
+      <c r="B18" s="47" t="s">
         <v>59</v>
       </c>
-      <c r="C18" s="46" t="s">
+      <c r="C18" s="47" t="s">
         <v>7</v>
       </c>
-      <c r="D18" s="46" t="s">
+      <c r="D18" s="47" t="s">
         <v>56</v>
       </c>
-      <c r="E18" s="46" t="s">
+      <c r="E18" s="47" t="s">
         <v>60</v>
       </c>
     </row>
     <row r="19" spans="1:5">
-      <c r="A19" s="48" t="s">
+      <c r="A19" s="49" t="s">
         <v>61</v>
       </c>
-      <c r="B19" s="46" t="s">
+      <c r="B19" s="47" t="s">
         <v>62</v>
       </c>
-      <c r="C19" s="46" t="s">
+      <c r="C19" s="47" t="s">
         <v>18</v>
       </c>
-      <c r="D19" s="46" t="s">
+      <c r="D19" s="47" t="s">
         <v>63</v>
       </c>
-      <c r="E19" s="46" t="s">
+      <c r="E19" s="47" t="s">
         <v>64</v>
       </c>
     </row>
@@ -5288,7 +5335,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr filterMode="1"/>
-  <dimension ref="A1:G113"/>
+  <dimension ref="A1:G114"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5" outlineLevelCol="6"/>
   <cols>
     <col min="1" max="1" width="15.8" customWidth="1"/>
@@ -5372,7 +5419,7 @@
       </c>
       <c r="G5" s="2"/>
     </row>
-    <row r="6" ht="27" hidden="1" spans="1:7">
+    <row r="6" ht="27" spans="1:7">
       <c r="A6" s="2" t="s">
         <v>81</v>
       </c>
@@ -5410,7 +5457,7 @@
       <c r="F7" s="2"/>
       <c r="G7" s="2"/>
     </row>
-    <row r="8" ht="16.5" hidden="1" spans="1:7">
+    <row r="8" ht="16.5" spans="1:7">
       <c r="A8" s="2" t="s">
         <v>89</v>
       </c>
@@ -5431,7 +5478,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="9" ht="135" hidden="1" spans="1:7">
+    <row r="9" ht="135" spans="1:7">
       <c r="A9" s="2" t="s">
         <v>92</v>
       </c>
@@ -6610,11 +6657,11 @@
         <v>19</v>
       </c>
     </row>
-    <row r="72" ht="27" spans="1:7">
+    <row r="72" ht="27" hidden="1" spans="1:7">
       <c r="A72" s="2" t="s">
         <v>293</v>
       </c>
-      <c r="B72" s="29" t="s">
+      <c r="B72" s="28" t="s">
         <v>294</v>
       </c>
       <c r="C72" s="27" t="s">
@@ -6626,49 +6673,53 @@
       <c r="E72" s="27" t="s">
         <v>79</v>
       </c>
-      <c r="F72" s="2"/>
+      <c r="F72" s="2" t="s">
+        <v>80</v>
+      </c>
       <c r="G72" s="2"/>
     </row>
-    <row r="73" ht="19.5" hidden="1" spans="1:7">
-      <c r="A73" s="2"/>
+    <row r="73" ht="54" spans="1:7">
+      <c r="A73" s="2" t="s">
+        <v>297</v>
+      </c>
       <c r="B73" s="35" t="s">
-        <v>297</v>
-      </c>
-      <c r="C73" s="2"/>
-      <c r="D73" s="26"/>
+        <v>298</v>
+      </c>
+      <c r="C73" s="27" t="s">
+        <v>295</v>
+      </c>
+      <c r="D73" s="29" t="s">
+        <v>299</v>
+      </c>
       <c r="E73" s="27" t="s">
-        <v>74</v>
+        <v>79</v>
       </c>
       <c r="F73" s="2"/>
       <c r="G73" s="2"/>
     </row>
-    <row r="74" ht="30" hidden="1" spans="1:7">
+    <row r="74" ht="19.5" hidden="1" spans="1:7">
       <c r="A74" s="2"/>
-      <c r="B74" s="27" t="s">
-        <v>298</v>
-      </c>
-      <c r="C74" s="29" t="s">
-        <v>295</v>
-      </c>
-      <c r="D74" s="29" t="s">
-        <v>299</v>
-      </c>
+      <c r="B74" s="36" t="s">
+        <v>300</v>
+      </c>
+      <c r="C74" s="2"/>
+      <c r="D74" s="26"/>
       <c r="E74" s="27" t="s">
-        <v>88</v>
+        <v>74</v>
       </c>
       <c r="F74" s="2"/>
       <c r="G74" s="2"/>
     </row>
-    <row r="75" ht="27" hidden="1" spans="1:7">
+    <row r="75" ht="30" hidden="1" spans="1:7">
       <c r="A75" s="2"/>
       <c r="B75" s="27" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="C75" s="29" t="s">
         <v>295</v>
       </c>
-      <c r="D75" s="27" t="s">
-        <v>301</v>
+      <c r="D75" s="29" t="s">
+        <v>302</v>
       </c>
       <c r="E75" s="27" t="s">
         <v>88</v>
@@ -6676,22 +6727,28 @@
       <c r="F75" s="2"/>
       <c r="G75" s="2"/>
     </row>
-    <row r="76" ht="19.5" hidden="1" spans="1:7">
+    <row r="76" ht="27" hidden="1" spans="1:7">
       <c r="A76" s="2"/>
-      <c r="B76" s="35" t="s">
-        <v>302</v>
-      </c>
-      <c r="C76" s="2"/>
-      <c r="D76" s="26"/>
+      <c r="B76" s="27" t="s">
+        <v>303</v>
+      </c>
+      <c r="C76" s="29" t="s">
+        <v>295</v>
+      </c>
+      <c r="D76" s="27" t="s">
+        <v>304</v>
+      </c>
       <c r="E76" s="27" t="s">
-        <v>74</v>
+        <v>88</v>
       </c>
       <c r="F76" s="2"/>
       <c r="G76" s="2"/>
     </row>
-    <row r="77" ht="16.5" hidden="1" spans="1:7">
+    <row r="77" ht="19.5" hidden="1" spans="1:7">
       <c r="A77" s="2"/>
-      <c r="B77" s="2"/>
+      <c r="B77" s="36" t="s">
+        <v>305</v>
+      </c>
       <c r="C77" s="2"/>
       <c r="D77" s="26"/>
       <c r="E77" s="27" t="s">
@@ -6700,11 +6757,9 @@
       <c r="F77" s="2"/>
       <c r="G77" s="2"/>
     </row>
-    <row r="78" ht="19.5" hidden="1" spans="1:7">
+    <row r="78" ht="16.5" hidden="1" spans="1:7">
       <c r="A78" s="2"/>
-      <c r="B78" s="35" t="s">
-        <v>303</v>
-      </c>
+      <c r="B78" s="2"/>
       <c r="C78" s="2"/>
       <c r="D78" s="26"/>
       <c r="E78" s="27" t="s">
@@ -6713,31 +6768,29 @@
       <c r="F78" s="2"/>
       <c r="G78" s="2"/>
     </row>
-    <row r="79" ht="67.5" hidden="1" spans="1:7">
+    <row r="79" ht="19.5" hidden="1" spans="1:7">
       <c r="A79" s="2"/>
-      <c r="B79" s="26" t="s">
-        <v>304</v>
-      </c>
-      <c r="C79" s="2" t="s">
-        <v>192</v>
-      </c>
-      <c r="D79" s="26" t="s">
-        <v>305</v>
-      </c>
+      <c r="B79" s="36" t="s">
+        <v>306</v>
+      </c>
+      <c r="C79" s="2"/>
+      <c r="D79" s="26"/>
       <c r="E79" s="27" t="s">
-        <v>88</v>
+        <v>74</v>
       </c>
       <c r="F79" s="2"/>
       <c r="G79" s="2"/>
     </row>
-    <row r="80" ht="16.5" hidden="1" spans="1:7">
+    <row r="80" ht="67.5" hidden="1" spans="1:7">
       <c r="A80" s="2"/>
-      <c r="B80" s="27" t="s">
-        <v>306</v>
-      </c>
-      <c r="C80" s="27"/>
-      <c r="D80" s="27" t="s">
+      <c r="B80" s="26" t="s">
         <v>307</v>
+      </c>
+      <c r="C80" s="2" t="s">
+        <v>192</v>
+      </c>
+      <c r="D80" s="26" t="s">
+        <v>308</v>
       </c>
       <c r="E80" s="27" t="s">
         <v>88</v>
@@ -6745,52 +6798,52 @@
       <c r="F80" s="2"/>
       <c r="G80" s="2"/>
     </row>
-    <row r="81" ht="27" hidden="1" spans="1:7">
-      <c r="A81" s="2" t="s">
-        <v>308</v>
-      </c>
-      <c r="B81" s="36" t="s">
+    <row r="81" ht="16.5" hidden="1" spans="1:7">
+      <c r="A81" s="2"/>
+      <c r="B81" s="27" t="s">
         <v>309</v>
       </c>
-      <c r="C81" s="27" t="s">
+      <c r="C81" s="27"/>
+      <c r="D81" s="27" t="s">
         <v>310</v>
       </c>
-      <c r="D81" s="27" t="s">
+      <c r="E81" s="27" t="s">
+        <v>88</v>
+      </c>
+      <c r="F81" s="2"/>
+      <c r="G81" s="2"/>
+    </row>
+    <row r="82" ht="27" hidden="1" spans="1:7">
+      <c r="A82" s="2" t="s">
         <v>311</v>
       </c>
-      <c r="E81" s="27" t="s">
+      <c r="B82" s="37" t="s">
+        <v>312</v>
+      </c>
+      <c r="C82" s="27" t="s">
+        <v>313</v>
+      </c>
+      <c r="D82" s="27" t="s">
+        <v>314</v>
+      </c>
+      <c r="E82" s="27" t="s">
         <v>79</v>
       </c>
-      <c r="F81" s="2" t="s">
+      <c r="F82" s="2" t="s">
         <v>80</v>
       </c>
-      <c r="G81" s="2"/>
-    </row>
-    <row r="82" ht="16.5" hidden="1" spans="1:7">
-      <c r="A82" s="2"/>
-      <c r="B82" s="2" t="s">
-        <v>312</v>
-      </c>
-      <c r="C82" s="2" t="s">
-        <v>313</v>
-      </c>
-      <c r="D82" s="26">
-        <v>742830</v>
-      </c>
-      <c r="E82" s="27" t="s">
-        <v>88</v>
-      </c>
-      <c r="F82" s="2"/>
       <c r="G82" s="2"/>
     </row>
-    <row r="83" ht="27" hidden="1" spans="1:7">
+    <row r="83" ht="16.5" hidden="1" spans="1:7">
       <c r="A83" s="2"/>
       <c r="B83" s="2" t="s">
-        <v>314</v>
-      </c>
-      <c r="C83" s="2"/>
-      <c r="D83" s="26" t="s">
         <v>315</v>
+      </c>
+      <c r="C83" s="2" t="s">
+        <v>316</v>
+      </c>
+      <c r="D83" s="26">
+        <v>742830</v>
       </c>
       <c r="E83" s="27" t="s">
         <v>88</v>
@@ -6798,11 +6851,9 @@
       <c r="F83" s="2"/>
       <c r="G83" s="2"/>
     </row>
-    <row r="84" ht="16.5" hidden="1" spans="1:7">
-      <c r="A84" s="37" t="s">
-        <v>316</v>
-      </c>
-      <c r="B84" s="38" t="s">
+    <row r="84" ht="27" hidden="1" spans="1:7">
+      <c r="A84" s="2"/>
+      <c r="B84" s="2" t="s">
         <v>317</v>
       </c>
       <c r="C84" s="2"/>
@@ -6810,23 +6861,19 @@
         <v>318</v>
       </c>
       <c r="E84" s="27" t="s">
-        <v>79</v>
-      </c>
-      <c r="F84" s="2" t="s">
-        <v>80</v>
-      </c>
+        <v>88</v>
+      </c>
+      <c r="F84" s="2"/>
       <c r="G84" s="2"/>
     </row>
-    <row r="85" ht="54" hidden="1" spans="1:7">
-      <c r="A85" s="37" t="s">
+    <row r="85" ht="16.5" hidden="1" spans="1:7">
+      <c r="A85" s="38" t="s">
         <v>319</v>
       </c>
-      <c r="B85" s="38" t="s">
+      <c r="B85" s="39" t="s">
         <v>320</v>
       </c>
-      <c r="C85" s="2" t="s">
-        <v>126</v>
-      </c>
+      <c r="C85" s="2"/>
       <c r="D85" s="26" t="s">
         <v>321</v>
       </c>
@@ -6838,18 +6885,18 @@
       </c>
       <c r="G85" s="2"/>
     </row>
-    <row r="86" ht="16.5" hidden="1" spans="1:7">
-      <c r="A86" s="2" t="s">
+    <row r="86" ht="54" hidden="1" spans="1:7">
+      <c r="A86" s="38" t="s">
         <v>322</v>
       </c>
-      <c r="B86" s="38" t="s">
+      <c r="B86" s="39" t="s">
         <v>323</v>
       </c>
       <c r="C86" s="2" t="s">
+        <v>126</v>
+      </c>
+      <c r="D86" s="26" t="s">
         <v>324</v>
-      </c>
-      <c r="D86" s="26" t="s">
-        <v>325</v>
       </c>
       <c r="E86" s="27" t="s">
         <v>79</v>
@@ -6859,50 +6906,56 @@
       </c>
       <c r="G86" s="2"/>
     </row>
-    <row r="87" ht="54" hidden="1" spans="1:7">
+    <row r="87" ht="16.5" hidden="1" spans="1:7">
       <c r="A87" s="2" t="s">
+        <v>325</v>
+      </c>
+      <c r="B87" s="39" t="s">
         <v>326</v>
       </c>
-      <c r="B87" s="2" t="s">
+      <c r="C87" s="2" t="s">
         <v>327</v>
       </c>
-      <c r="C87" s="2" t="s">
+      <c r="D87" s="26" t="s">
         <v>328</v>
       </c>
-      <c r="D87" s="26" t="s">
+      <c r="E87" s="27" t="s">
+        <v>79</v>
+      </c>
+      <c r="F87" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="G87" s="2"/>
+    </row>
+    <row r="88" ht="54" hidden="1" spans="1:7">
+      <c r="A88" s="2" t="s">
         <v>329</v>
       </c>
-      <c r="E87" s="27" t="s">
-        <v>99</v>
-      </c>
-      <c r="F87" s="2"/>
-      <c r="G87" s="2">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="88" ht="54" hidden="1" spans="1:7">
-      <c r="A88" s="2"/>
       <c r="B88" s="2" t="s">
         <v>330</v>
       </c>
-      <c r="C88" s="2"/>
+      <c r="C88" s="2" t="s">
+        <v>331</v>
+      </c>
       <c r="D88" s="26" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="E88" s="27" t="s">
-        <v>88</v>
+        <v>99</v>
       </c>
       <c r="F88" s="2"/>
-      <c r="G88" s="2"/>
-    </row>
-    <row r="89" ht="81" hidden="1" spans="1:7">
+      <c r="G88" s="2">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="89" ht="54" hidden="1" spans="1:7">
       <c r="A89" s="2"/>
-      <c r="B89" s="26" t="s">
-        <v>332</v>
+      <c r="B89" s="2" t="s">
+        <v>333</v>
       </c>
       <c r="C89" s="2"/>
       <c r="D89" s="26" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="E89" s="27" t="s">
         <v>88</v>
@@ -6910,152 +6963,150 @@
       <c r="F89" s="2"/>
       <c r="G89" s="2"/>
     </row>
-    <row r="90" ht="16.5" hidden="1" spans="1:7">
-      <c r="A90" s="2" t="s">
-        <v>334</v>
-      </c>
-      <c r="B90" s="39" t="s">
+    <row r="90" ht="81" hidden="1" spans="1:7">
+      <c r="A90" s="2"/>
+      <c r="B90" s="26" t="s">
         <v>335</v>
       </c>
-      <c r="C90" s="2" t="s">
-        <v>83</v>
-      </c>
+      <c r="C90" s="2"/>
       <c r="D90" s="26" t="s">
         <v>336</v>
       </c>
       <c r="E90" s="27" t="s">
+        <v>88</v>
+      </c>
+      <c r="F90" s="2"/>
+      <c r="G90" s="2"/>
+    </row>
+    <row r="91" ht="16.5" hidden="1" spans="1:7">
+      <c r="A91" s="2" t="s">
+        <v>337</v>
+      </c>
+      <c r="B91" s="40" t="s">
+        <v>338</v>
+      </c>
+      <c r="C91" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="D91" s="26" t="s">
+        <v>339</v>
+      </c>
+      <c r="E91" s="27" t="s">
         <v>79</v>
       </c>
-      <c r="F90" s="2" t="s">
+      <c r="F91" s="2" t="s">
         <v>80</v>
       </c>
-      <c r="G90" s="2"/>
-    </row>
-    <row r="91" ht="27" hidden="1" spans="1:7">
-      <c r="A91" s="2"/>
-      <c r="B91" s="2" t="s">
-        <v>337</v>
-      </c>
-      <c r="C91" s="2"/>
-      <c r="D91" s="26" t="s">
-        <v>338</v>
-      </c>
-      <c r="E91" s="27" t="s">
+      <c r="G91" s="2"/>
+    </row>
+    <row r="92" ht="27" hidden="1" spans="1:7">
+      <c r="A92" s="2"/>
+      <c r="B92" s="2" t="s">
+        <v>340</v>
+      </c>
+      <c r="C92" s="2"/>
+      <c r="D92" s="26" t="s">
+        <v>341</v>
+      </c>
+      <c r="E92" s="27" t="s">
         <v>88</v>
       </c>
-      <c r="F91" s="2"/>
-      <c r="G91" s="2"/>
-    </row>
-    <row r="92" ht="30" hidden="1" spans="1:7">
-      <c r="A92" s="2" t="s">
-        <v>339</v>
-      </c>
-      <c r="B92" s="27" t="s">
-        <v>340</v>
-      </c>
-      <c r="C92" s="29" t="s">
-        <v>283</v>
-      </c>
-      <c r="D92" s="27" t="s">
-        <v>341</v>
-      </c>
-      <c r="E92" s="27" t="s">
-        <v>99</v>
-      </c>
       <c r="F92" s="2"/>
-      <c r="G92" s="2">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="93" ht="81" hidden="1" spans="1:7">
+      <c r="G92" s="2"/>
+    </row>
+    <row r="93" ht="30" hidden="1" spans="1:7">
       <c r="A93" s="2" t="s">
         <v>342</v>
       </c>
-      <c r="B93" s="39" t="s">
+      <c r="B93" s="27" t="s">
         <v>343</v>
       </c>
-      <c r="C93" s="2" t="s">
+      <c r="C93" s="29" t="s">
+        <v>283</v>
+      </c>
+      <c r="D93" s="27" t="s">
         <v>344</v>
       </c>
-      <c r="D93" s="26" t="s">
+      <c r="E93" s="27" t="s">
+        <v>99</v>
+      </c>
+      <c r="F93" s="2"/>
+      <c r="G93" s="2">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="94" ht="81" hidden="1" spans="1:7">
+      <c r="A94" s="2" t="s">
         <v>345</v>
       </c>
-      <c r="E93" s="27" t="s">
+      <c r="B94" s="40" t="s">
+        <v>346</v>
+      </c>
+      <c r="C94" s="2" t="s">
+        <v>347</v>
+      </c>
+      <c r="D94" s="26" t="s">
+        <v>348</v>
+      </c>
+      <c r="E94" s="27" t="s">
         <v>79</v>
       </c>
-      <c r="F93" s="2" t="s">
+      <c r="F94" s="2" t="s">
         <v>80</v>
       </c>
-      <c r="G93" s="2"/>
-    </row>
-    <row r="94" ht="57" hidden="1" spans="1:7">
-      <c r="A94" s="2" t="s">
-        <v>346</v>
-      </c>
-      <c r="B94" s="27" t="s">
+      <c r="G94" s="2"/>
+    </row>
+    <row r="95" ht="57" hidden="1" spans="1:7">
+      <c r="A95" s="2" t="s">
+        <v>349</v>
+      </c>
+      <c r="B95" s="27" t="s">
+        <v>350</v>
+      </c>
+      <c r="C95" s="29" t="s">
+        <v>351</v>
+      </c>
+      <c r="D95" s="27" t="s">
+        <v>352</v>
+      </c>
+      <c r="E95" s="27" t="s">
+        <v>99</v>
+      </c>
+      <c r="F95" s="2"/>
+      <c r="G95" s="2">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="96" customFormat="1" ht="27" hidden="1" spans="1:7">
+      <c r="A96" s="2" t="s">
+        <v>353</v>
+      </c>
+      <c r="B96" s="40" t="s">
+        <v>354</v>
+      </c>
+      <c r="C96" s="2" t="s">
         <v>347</v>
       </c>
-      <c r="C94" s="29" t="s">
-        <v>348</v>
-      </c>
-      <c r="D94" s="27" t="s">
-        <v>349</v>
-      </c>
-      <c r="E94" s="27" t="s">
-        <v>99</v>
-      </c>
-      <c r="F94" s="2"/>
-      <c r="G94" s="2">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="95" customFormat="1" ht="27" hidden="1" spans="1:7">
-      <c r="A95" s="2" t="s">
-        <v>350</v>
-      </c>
-      <c r="B95" s="39" t="s">
-        <v>351</v>
-      </c>
-      <c r="C95" s="2" t="s">
-        <v>344</v>
-      </c>
-      <c r="D95" s="26" t="s">
-        <v>352</v>
-      </c>
-      <c r="E95" s="2" t="s">
+      <c r="D96" s="26" t="s">
+        <v>355</v>
+      </c>
+      <c r="E96" s="2" t="s">
         <v>79</v>
       </c>
-      <c r="F95" s="2" t="s">
+      <c r="F96" s="2" t="s">
         <v>80</v>
       </c>
-      <c r="G95" s="2"/>
-    </row>
-    <row r="96" customFormat="1" ht="40.5" hidden="1" spans="1:7">
-      <c r="A96" s="2"/>
-      <c r="B96" s="2" t="s">
-        <v>353</v>
-      </c>
-      <c r="C96" s="2" t="s">
-        <v>94</v>
-      </c>
-      <c r="D96" s="26" t="s">
-        <v>354</v>
-      </c>
-      <c r="E96" s="2" t="s">
-        <v>88</v>
-      </c>
-      <c r="F96" s="2"/>
       <c r="G96" s="2"/>
     </row>
-    <row r="97" customFormat="1" hidden="1" spans="1:7">
+    <row r="97" customFormat="1" ht="40.5" hidden="1" spans="1:7">
       <c r="A97" s="2"/>
       <c r="B97" s="2" t="s">
-        <v>355</v>
+        <v>356</v>
       </c>
       <c r="C97" s="2" t="s">
-        <v>356</v>
-      </c>
-      <c r="D97" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="D97" s="26" t="s">
         <v>357</v>
       </c>
       <c r="E97" s="2" t="s">
@@ -7064,51 +7115,49 @@
       <c r="F97" s="2"/>
       <c r="G97" s="2"/>
     </row>
-    <row r="98" customFormat="1" ht="40.5" hidden="1" spans="1:7">
-      <c r="A98" s="2" t="s">
+    <row r="98" customFormat="1" hidden="1" spans="1:7">
+      <c r="A98" s="2"/>
+      <c r="B98" s="2" t="s">
         <v>358</v>
       </c>
-      <c r="B98" s="26" t="s">
+      <c r="C98" s="2" t="s">
         <v>359</v>
       </c>
-      <c r="C98" s="2" t="s">
+      <c r="D98" s="2" t="s">
+        <v>360</v>
+      </c>
+      <c r="E98" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="F98" s="2"/>
+      <c r="G98" s="2"/>
+    </row>
+    <row r="99" customFormat="1" ht="40.5" hidden="1" spans="1:7">
+      <c r="A99" s="2" t="s">
+        <v>361</v>
+      </c>
+      <c r="B99" s="26" t="s">
+        <v>362</v>
+      </c>
+      <c r="C99" s="2" t="s">
         <v>83</v>
       </c>
-      <c r="D98" s="26" t="s">
-        <v>360</v>
-      </c>
-      <c r="E98" s="2" t="s">
-        <v>99</v>
-      </c>
-      <c r="F98" s="2"/>
-      <c r="G98" s="2">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="99" customFormat="1" ht="67.5" hidden="1" spans="1:7">
-      <c r="A99" s="40" t="s">
-        <v>361</v>
-      </c>
-      <c r="B99" s="41" t="s">
-        <v>362</v>
-      </c>
-      <c r="C99" s="2"/>
       <c r="D99" s="26" t="s">
         <v>363</v>
       </c>
       <c r="E99" s="2" t="s">
-        <v>79</v>
-      </c>
-      <c r="F99" s="2" t="s">
-        <v>80</v>
-      </c>
-      <c r="G99" s="2"/>
-    </row>
-    <row r="100" customFormat="1" ht="54" hidden="1" spans="1:7">
-      <c r="A100" s="40" t="s">
+        <v>99</v>
+      </c>
+      <c r="F99" s="2"/>
+      <c r="G99" s="2">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="100" customFormat="1" ht="67.5" hidden="1" spans="1:7">
+      <c r="A100" s="41" t="s">
         <v>364</v>
       </c>
-      <c r="B100" s="39" t="s">
+      <c r="B100" s="42" t="s">
         <v>365</v>
       </c>
       <c r="C100" s="2"/>
@@ -7123,92 +7172,104 @@
       </c>
       <c r="G100" s="2"/>
     </row>
-    <row r="101" customFormat="1" ht="67.5" hidden="1" spans="1:7">
-      <c r="A101" s="2" t="s">
+    <row r="101" customFormat="1" ht="54" hidden="1" spans="1:7">
+      <c r="A101" s="41" t="s">
         <v>367</v>
       </c>
-      <c r="B101" s="2" t="s">
+      <c r="B101" s="40" t="s">
         <v>368</v>
       </c>
-      <c r="C101" s="2" t="s">
+      <c r="C101" s="2"/>
+      <c r="D101" s="26" t="s">
         <v>369</v>
       </c>
-      <c r="D101" s="26" t="s">
+      <c r="E101" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="F101" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="G101" s="2"/>
+    </row>
+    <row r="102" customFormat="1" ht="67.5" hidden="1" spans="1:7">
+      <c r="A102" s="2" t="s">
         <v>370</v>
       </c>
-      <c r="E101" s="2" t="s">
+      <c r="B102" s="2" t="s">
+        <v>371</v>
+      </c>
+      <c r="C102" s="2" t="s">
+        <v>372</v>
+      </c>
+      <c r="D102" s="26" t="s">
+        <v>373</v>
+      </c>
+      <c r="E102" s="2" t="s">
         <v>99</v>
       </c>
-      <c r="F101" s="2" t="s">
-        <v>371</v>
-      </c>
-      <c r="G101" s="2"/>
-    </row>
-    <row r="102" customFormat="1" ht="54" hidden="1" spans="1:7">
-      <c r="A102" s="2" t="s">
-        <v>372</v>
-      </c>
-      <c r="B102" s="2" t="s">
-        <v>373</v>
-      </c>
-      <c r="C102" s="2" t="s">
+      <c r="F102" s="2" t="s">
         <v>374</v>
-      </c>
-      <c r="D102" s="26" t="s">
-        <v>375</v>
-      </c>
-      <c r="E102" s="2" t="s">
-        <v>88</v>
-      </c>
-      <c r="F102" s="2" t="s">
-        <v>371</v>
       </c>
       <c r="G102" s="2"/>
     </row>
     <row r="103" customFormat="1" ht="54" hidden="1" spans="1:7">
       <c r="A103" s="2" t="s">
+        <v>375</v>
+      </c>
+      <c r="B103" s="2" t="s">
         <v>376</v>
       </c>
-      <c r="B103" s="2" t="s">
+      <c r="C103" s="2" t="s">
         <v>377</v>
       </c>
-      <c r="C103" s="2" t="s">
+      <c r="D103" s="26" t="s">
         <v>378</v>
       </c>
-      <c r="D103" s="26" t="s">
+      <c r="E103" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="F103" s="2" t="s">
+        <v>374</v>
+      </c>
+      <c r="G103" s="2"/>
+    </row>
+    <row r="104" customFormat="1" ht="54" hidden="1" spans="1:7">
+      <c r="A104" s="2" t="s">
         <v>379</v>
       </c>
-      <c r="E103" s="2" t="s">
-        <v>79</v>
-      </c>
-      <c r="F103" s="2" t="s">
-        <v>371</v>
-      </c>
-      <c r="G103" s="2"/>
-    </row>
-    <row r="104" customFormat="1" ht="40.5" spans="1:7">
-      <c r="A104" s="2" t="s">
+      <c r="B104" s="40" t="s">
         <v>380</v>
       </c>
-      <c r="B104" s="2" t="s">
+      <c r="C104" s="2" t="s">
         <v>381</v>
-      </c>
-      <c r="C104" s="27" t="s">
-        <v>295</v>
       </c>
       <c r="D104" s="26" t="s">
         <v>382</v>
       </c>
       <c r="E104" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="F104" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="G104" s="2"/>
+    </row>
+    <row r="105" customFormat="1" ht="40.5" hidden="1" spans="1:7">
+      <c r="A105" s="2" t="s">
+        <v>383</v>
+      </c>
+      <c r="B105" s="2" t="s">
+        <v>384</v>
+      </c>
+      <c r="C105" s="27" t="s">
+        <v>295</v>
+      </c>
+      <c r="D105" s="26" t="s">
+        <v>385</v>
+      </c>
+      <c r="E105" s="2" t="s">
         <v>99</v>
       </c>
-    </row>
-    <row r="105" customFormat="1" spans="1:7">
-      <c r="A105" s="2"/>
-      <c r="B105" s="2"/>
-      <c r="C105" s="2"/>
-      <c r="D105" s="26"/>
-      <c r="E105" s="2"/>
     </row>
     <row r="106" customFormat="1" spans="1:7">
       <c r="A106" s="2"/>
@@ -7217,32 +7278,42 @@
       <c r="D106" s="26"/>
       <c r="E106" s="2"/>
     </row>
-    <row r="110" ht="19.5" spans="1:7">
-      <c r="B110" s="42" t="s">
-        <v>383</v>
-      </c>
-    </row>
-    <row r="111" ht="17.25" spans="1:7">
+    <row r="107" customFormat="1" spans="1:7">
+      <c r="A107" s="2"/>
+      <c r="B107" s="2"/>
+      <c r="C107" s="2"/>
+      <c r="D107" s="26"/>
+      <c r="E107" s="2"/>
+    </row>
+    <row r="111" ht="19.5" spans="1:7">
       <c r="B111" s="43" t="s">
-        <v>384</v>
+        <v>386</v>
       </c>
     </row>
     <row r="112" ht="17.25" spans="1:7">
-      <c r="B112" s="43" t="s">
-        <v>385</v>
+      <c r="B112" s="44" t="s">
+        <v>387</v>
       </c>
     </row>
     <row r="113" ht="17.25" spans="2:2">
-      <c r="B113" s="43" t="s">
-        <v>386</v>
+      <c r="B113" s="44" t="s">
+        <v>388</v>
+      </c>
+    </row>
+    <row r="114" ht="17.25" spans="2:2">
+      <c r="B114" s="44" t="s">
+        <v>389</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" ref="A3:G104" etc:filterBottomFollowUsedRange="0">
-    <filterColumn colId="1">
+  <autoFilter xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" ref="A3:G105" etc:filterBottomFollowUsedRange="0">
+    <filterColumn colId="4">
       <filters>
-        <filter val="CLI&gt;GUI界面迁移"/>
+        <filter val="P0"/>
       </filters>
+    </filterColumn>
+    <filterColumn colId="5">
+      <filters blank="1"/>
     </filterColumn>
     <extLst/>
   </autoFilter>
@@ -7269,12 +7340,12 @@
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" t="s">
-        <v>387</v>
+        <v>390</v>
       </c>
     </row>
     <row r="2" ht="29.6" customHeight="1" spans="1:2">
       <c r="A2" t="s">
-        <v>388</v>
+        <v>391</v>
       </c>
     </row>
     <row r="3" spans="1:2">
@@ -7282,7 +7353,7 @@
         <v>1</v>
       </c>
       <c r="B3" t="s">
-        <v>389</v>
+        <v>392</v>
       </c>
     </row>
     <row r="4" spans="1:2">
@@ -7290,7 +7361,7 @@
         <v>2</v>
       </c>
       <c r="B4" t="s">
-        <v>390</v>
+        <v>393</v>
       </c>
     </row>
     <row r="5" spans="1:2">
@@ -7298,7 +7369,7 @@
         <v>3</v>
       </c>
       <c r="B5" t="s">
-        <v>391</v>
+        <v>394</v>
       </c>
     </row>
     <row r="6" spans="1:2">
@@ -7306,7 +7377,7 @@
         <v>4</v>
       </c>
       <c r="B6" t="s">
-        <v>392</v>
+        <v>395</v>
       </c>
     </row>
     <row r="7" spans="1:2">
@@ -7314,7 +7385,7 @@
         <v>5</v>
       </c>
       <c r="B7" t="s">
-        <v>393</v>
+        <v>396</v>
       </c>
     </row>
     <row r="8" spans="1:2">
@@ -7322,7 +7393,7 @@
         <v>6</v>
       </c>
       <c r="B8" t="s">
-        <v>394</v>
+        <v>397</v>
       </c>
     </row>
     <row r="9" spans="1:2">
@@ -7330,7 +7401,7 @@
         <v>7</v>
       </c>
       <c r="B9" t="s">
-        <v>395</v>
+        <v>398</v>
       </c>
     </row>
     <row r="10" spans="1:2">
@@ -7338,7 +7409,7 @@
         <v>8</v>
       </c>
       <c r="B10" t="s">
-        <v>396</v>
+        <v>399</v>
       </c>
     </row>
     <row r="11" spans="1:2">
@@ -7346,7 +7417,7 @@
         <v>9</v>
       </c>
       <c r="B11" t="s">
-        <v>397</v>
+        <v>400</v>
       </c>
     </row>
     <row r="12" spans="1:2">
@@ -7354,7 +7425,7 @@
         <v>10</v>
       </c>
       <c r="B12" t="s">
-        <v>398</v>
+        <v>401</v>
       </c>
     </row>
     <row r="13" spans="1:2">
@@ -7362,7 +7433,7 @@
         <v>11</v>
       </c>
       <c r="B13" t="s">
-        <v>399</v>
+        <v>402</v>
       </c>
     </row>
     <row r="14" spans="1:2">
@@ -7370,7 +7441,7 @@
         <v>12</v>
       </c>
       <c r="B14" t="s">
-        <v>400</v>
+        <v>403</v>
       </c>
     </row>
     <row r="15" spans="1:2">
@@ -7378,7 +7449,7 @@
         <v>13</v>
       </c>
       <c r="B15" t="s">
-        <v>401</v>
+        <v>404</v>
       </c>
     </row>
     <row r="16" spans="1:2">
@@ -7386,7 +7457,7 @@
         <v>14</v>
       </c>
       <c r="B16" t="s">
-        <v>402</v>
+        <v>405</v>
       </c>
     </row>
     <row r="17" spans="1:2">
@@ -7394,7 +7465,7 @@
         <v>15</v>
       </c>
       <c r="B17" t="s">
-        <v>403</v>
+        <v>406</v>
       </c>
     </row>
     <row r="18" spans="1:2">
@@ -7402,7 +7473,7 @@
         <v>16</v>
       </c>
       <c r="B18" t="s">
-        <v>404</v>
+        <v>407</v>
       </c>
     </row>
     <row r="19" spans="1:2">
@@ -7410,7 +7481,7 @@
         <v>17</v>
       </c>
       <c r="B19" t="s">
-        <v>405</v>
+        <v>408</v>
       </c>
     </row>
     <row r="20" spans="1:2">
@@ -7418,7 +7489,7 @@
         <v>18</v>
       </c>
       <c r="B20" t="s">
-        <v>406</v>
+        <v>409</v>
       </c>
     </row>
     <row r="21" spans="1:2">
@@ -7426,7 +7497,7 @@
         <v>19</v>
       </c>
       <c r="B21" t="s">
-        <v>407</v>
+        <v>410</v>
       </c>
     </row>
     <row r="22" spans="1:2">
@@ -7434,17 +7505,17 @@
         <v>20</v>
       </c>
       <c r="B22" t="s">
-        <v>408</v>
+        <v>411</v>
       </c>
     </row>
     <row r="24" spans="1:2">
       <c r="A24" t="s">
-        <v>409</v>
+        <v>412</v>
       </c>
     </row>
     <row r="25" spans="1:2">
       <c r="A25" t="s">
-        <v>388</v>
+        <v>391</v>
       </c>
     </row>
     <row r="26" spans="1:2">
@@ -7452,7 +7523,7 @@
         <v>1</v>
       </c>
       <c r="B26" t="s">
-        <v>410</v>
+        <v>413</v>
       </c>
     </row>
     <row r="27" spans="1:2">
@@ -7460,7 +7531,7 @@
         <v>2</v>
       </c>
       <c r="B27" t="s">
-        <v>411</v>
+        <v>414</v>
       </c>
     </row>
     <row r="28" spans="1:2">
@@ -7468,7 +7539,7 @@
         <v>3</v>
       </c>
       <c r="B28" t="s">
-        <v>412</v>
+        <v>415</v>
       </c>
     </row>
     <row r="29" spans="1:2">
@@ -7476,7 +7547,7 @@
         <v>4</v>
       </c>
       <c r="B29" t="s">
-        <v>413</v>
+        <v>416</v>
       </c>
     </row>
     <row r="30" spans="1:2">
@@ -7484,7 +7555,7 @@
         <v>5</v>
       </c>
       <c r="B30" t="s">
-        <v>414</v>
+        <v>417</v>
       </c>
     </row>
   </sheetData>
@@ -7507,186 +7578,186 @@
   <sheetData>
     <row r="1" spans="1:9">
       <c r="A1" s="15" t="s">
-        <v>415</v>
+        <v>418</v>
       </c>
       <c r="B1" s="16" t="s">
-        <v>416</v>
+        <v>419</v>
       </c>
       <c r="C1" s="16"/>
       <c r="D1" s="16"/>
       <c r="E1" s="16"/>
       <c r="F1" s="15" t="s">
-        <v>415</v>
+        <v>418</v>
       </c>
       <c r="G1" s="15" t="s">
-        <v>417</v>
+        <v>420</v>
       </c>
       <c r="H1" s="17"/>
       <c r="I1" s="15" t="s">
-        <v>418</v>
+        <v>421</v>
       </c>
     </row>
     <row r="2" spans="1:9">
       <c r="A2" s="15" t="s">
-        <v>419</v>
+        <v>422</v>
       </c>
       <c r="B2" s="15" t="s">
-        <v>420</v>
+        <v>423</v>
       </c>
       <c r="C2" s="15" t="s">
-        <v>421</v>
+        <v>424</v>
       </c>
       <c r="D2" s="15" t="s">
+        <v>425</v>
+      </c>
+      <c r="E2" s="15" t="s">
+        <v>426</v>
+      </c>
+      <c r="F2" s="15" t="s">
         <v>422</v>
       </c>
-      <c r="E2" s="15" t="s">
-        <v>423</v>
-      </c>
-      <c r="F2" s="15" t="s">
-        <v>419</v>
-      </c>
       <c r="G2" s="15" t="s">
-        <v>421</v>
+        <v>424</v>
       </c>
       <c r="H2" s="15" t="s">
-        <v>423</v>
+        <v>426</v>
       </c>
       <c r="I2" s="18" t="s">
-        <v>424</v>
+        <v>427</v>
       </c>
     </row>
     <row r="3" spans="1:9">
       <c r="A3" s="15" t="s">
-        <v>425</v>
+        <v>428</v>
       </c>
       <c r="B3" s="15" t="s">
-        <v>426</v>
+        <v>429</v>
       </c>
       <c r="C3" s="15" t="s">
-        <v>426</v>
+        <v>429</v>
       </c>
       <c r="D3" s="15" t="s">
-        <v>427</v>
+        <v>430</v>
       </c>
       <c r="E3" s="15" t="s">
-        <v>427</v>
+        <v>430</v>
       </c>
       <c r="F3" s="15" t="s">
-        <v>425</v>
+        <v>428</v>
       </c>
       <c r="G3" s="15" t="s">
-        <v>428</v>
+        <v>431</v>
       </c>
       <c r="H3" s="15" t="s">
-        <v>428</v>
+        <v>431</v>
       </c>
       <c r="I3" s="18"/>
     </row>
     <row r="4" spans="1:9">
       <c r="A4" s="15" t="s">
-        <v>429</v>
+        <v>432</v>
       </c>
       <c r="B4" s="15" t="s">
+        <v>433</v>
+      </c>
+      <c r="C4" s="15" t="s">
+        <v>433</v>
+      </c>
+      <c r="D4" s="15" t="s">
+        <v>434</v>
+      </c>
+      <c r="E4" s="15" t="s">
         <v>430</v>
       </c>
-      <c r="C4" s="15" t="s">
-        <v>430</v>
-      </c>
-      <c r="D4" s="15" t="s">
-        <v>431</v>
-      </c>
-      <c r="E4" s="15" t="s">
-        <v>427</v>
-      </c>
       <c r="F4" s="15" t="s">
-        <v>429</v>
+        <v>432</v>
       </c>
       <c r="G4" s="15" t="s">
-        <v>430</v>
+        <v>433</v>
       </c>
       <c r="H4" s="15" t="s">
-        <v>431</v>
+        <v>434</v>
       </c>
       <c r="I4" s="18"/>
     </row>
     <row r="5" spans="1:9">
       <c r="A5" s="15" t="s">
-        <v>432</v>
+        <v>435</v>
       </c>
       <c r="B5" s="15" t="s">
-        <v>431</v>
+        <v>434</v>
       </c>
       <c r="C5" s="15" t="s">
-        <v>431</v>
+        <v>434</v>
       </c>
       <c r="D5" s="15" t="s">
-        <v>431</v>
+        <v>434</v>
       </c>
       <c r="E5" s="15" t="s">
-        <v>427</v>
+        <v>430</v>
       </c>
       <c r="F5" s="15" t="s">
-        <v>432</v>
+        <v>435</v>
       </c>
       <c r="G5" s="15" t="s">
-        <v>431</v>
+        <v>434</v>
       </c>
       <c r="H5" s="15" t="s">
-        <v>431</v>
+        <v>434</v>
       </c>
       <c r="I5" s="18"/>
     </row>
     <row r="6" spans="1:9">
       <c r="A6" s="15" t="s">
+        <v>436</v>
+      </c>
+      <c r="B6" s="15" t="s">
+        <v>434</v>
+      </c>
+      <c r="C6" s="15" t="s">
+        <v>434</v>
+      </c>
+      <c r="D6" s="15" t="s">
         <v>433</v>
       </c>
-      <c r="B6" s="15" t="s">
-        <v>431</v>
-      </c>
-      <c r="C6" s="15" t="s">
-        <v>431</v>
-      </c>
-      <c r="D6" s="15" t="s">
+      <c r="E6" s="15" t="s">
         <v>430</v>
       </c>
-      <c r="E6" s="15" t="s">
-        <v>427</v>
-      </c>
       <c r="F6" s="15" t="s">
+        <v>436</v>
+      </c>
+      <c r="G6" s="15" t="s">
+        <v>434</v>
+      </c>
+      <c r="H6" s="15" t="s">
         <v>433</v>
-      </c>
-      <c r="G6" s="15" t="s">
-        <v>431</v>
-      </c>
-      <c r="H6" s="15" t="s">
-        <v>430</v>
       </c>
       <c r="I6" s="18"/>
     </row>
     <row r="7" spans="1:9">
       <c r="A7" s="15" t="s">
-        <v>434</v>
+        <v>437</v>
       </c>
       <c r="B7" s="15" t="s">
-        <v>427</v>
+        <v>430</v>
       </c>
       <c r="C7" s="15" t="s">
-        <v>427</v>
+        <v>430</v>
       </c>
       <c r="D7" s="15" t="s">
-        <v>426</v>
+        <v>429</v>
       </c>
       <c r="E7" s="15" t="s">
-        <v>427</v>
+        <v>430</v>
       </c>
       <c r="F7" s="15" t="s">
-        <v>434</v>
+        <v>437</v>
       </c>
       <c r="G7" s="15" t="s">
-        <v>427</v>
+        <v>430</v>
       </c>
       <c r="H7" s="15" t="s">
-        <v>426</v>
+        <v>429</v>
       </c>
       <c r="I7" s="18"/>
     </row>
@@ -7703,255 +7774,255 @@
     </row>
     <row r="9" spans="1:9">
       <c r="A9" s="15" t="s">
-        <v>435</v>
+        <v>438</v>
       </c>
       <c r="B9" s="16" t="s">
-        <v>416</v>
+        <v>419</v>
       </c>
       <c r="C9" s="16"/>
       <c r="D9" s="16"/>
       <c r="E9" s="16"/>
       <c r="F9" s="15" t="s">
-        <v>435</v>
+        <v>438</v>
       </c>
       <c r="G9" s="15" t="s">
-        <v>417</v>
+        <v>420</v>
       </c>
       <c r="H9" s="17"/>
       <c r="I9" s="15" t="s">
-        <v>418</v>
+        <v>421</v>
       </c>
     </row>
     <row r="10" spans="1:9">
       <c r="A10" s="15" t="s">
-        <v>419</v>
+        <v>422</v>
       </c>
       <c r="B10" s="15" t="s">
-        <v>420</v>
+        <v>423</v>
       </c>
       <c r="C10" s="15" t="s">
-        <v>421</v>
+        <v>424</v>
       </c>
       <c r="D10" s="15" t="s">
+        <v>425</v>
+      </c>
+      <c r="E10" s="15" t="s">
+        <v>426</v>
+      </c>
+      <c r="F10" s="15" t="s">
         <v>422</v>
       </c>
-      <c r="E10" s="15" t="s">
-        <v>423</v>
-      </c>
-      <c r="F10" s="15" t="s">
-        <v>419</v>
-      </c>
       <c r="G10" s="15" t="s">
-        <v>421</v>
+        <v>424</v>
       </c>
       <c r="H10" s="15" t="s">
-        <v>423</v>
+        <v>426</v>
       </c>
       <c r="I10" s="18" t="s">
-        <v>436</v>
+        <v>439</v>
       </c>
     </row>
     <row r="11" spans="1:9">
       <c r="A11" s="15" t="s">
-        <v>425</v>
+        <v>428</v>
       </c>
       <c r="B11" s="15" t="s">
-        <v>426</v>
+        <v>429</v>
       </c>
       <c r="C11" s="17"/>
       <c r="D11" s="15" t="s">
-        <v>427</v>
+        <v>430</v>
       </c>
       <c r="E11" s="15" t="s">
-        <v>427</v>
+        <v>430</v>
       </c>
       <c r="F11" s="15" t="s">
-        <v>425</v>
+        <v>428</v>
       </c>
       <c r="G11" s="15" t="s">
-        <v>426</v>
+        <v>429</v>
       </c>
       <c r="H11" s="15" t="s">
-        <v>427</v>
+        <v>430</v>
       </c>
       <c r="I11" s="18"/>
     </row>
     <row r="12" spans="1:9">
       <c r="A12" s="15" t="s">
-        <v>429</v>
+        <v>432</v>
       </c>
       <c r="B12" s="15" t="s">
-        <v>430</v>
+        <v>433</v>
       </c>
       <c r="C12" s="17"/>
       <c r="D12" s="15" t="s">
-        <v>431</v>
+        <v>434</v>
       </c>
       <c r="E12" s="15" t="s">
-        <v>431</v>
+        <v>434</v>
       </c>
       <c r="F12" s="15" t="s">
-        <v>429</v>
+        <v>432</v>
       </c>
       <c r="G12" s="15" t="s">
-        <v>430</v>
+        <v>433</v>
       </c>
       <c r="H12" s="15" t="s">
-        <v>431</v>
+        <v>434</v>
       </c>
       <c r="I12" s="18"/>
     </row>
     <row r="13" spans="1:9">
       <c r="A13" s="15" t="s">
-        <v>432</v>
+        <v>435</v>
       </c>
       <c r="B13" s="15" t="s">
-        <v>431</v>
+        <v>434</v>
       </c>
       <c r="C13" s="17"/>
       <c r="D13" s="15" t="s">
-        <v>431</v>
+        <v>434</v>
       </c>
       <c r="E13" s="15" t="s">
-        <v>431</v>
+        <v>434</v>
       </c>
       <c r="F13" s="15" t="s">
-        <v>432</v>
+        <v>435</v>
       </c>
       <c r="G13" s="15" t="s">
-        <v>431</v>
+        <v>434</v>
       </c>
       <c r="H13" s="15" t="s">
-        <v>431</v>
+        <v>434</v>
       </c>
       <c r="I13" s="18"/>
     </row>
     <row r="14" spans="1:9">
       <c r="A14" s="15" t="s">
-        <v>433</v>
+        <v>436</v>
       </c>
       <c r="B14" s="15" t="s">
-        <v>431</v>
+        <v>434</v>
       </c>
       <c r="C14" s="17"/>
       <c r="D14" s="15" t="s">
-        <v>430</v>
+        <v>433</v>
       </c>
       <c r="E14" s="15" t="s">
-        <v>430</v>
+        <v>433</v>
       </c>
       <c r="F14" s="15" t="s">
+        <v>436</v>
+      </c>
+      <c r="G14" s="15" t="s">
+        <v>434</v>
+      </c>
+      <c r="H14" s="15" t="s">
         <v>433</v>
-      </c>
-      <c r="G14" s="15" t="s">
-        <v>431</v>
-      </c>
-      <c r="H14" s="15" t="s">
-        <v>430</v>
       </c>
       <c r="I14" s="18"/>
     </row>
     <row r="15" spans="1:9">
       <c r="A15" s="15" t="s">
-        <v>434</v>
+        <v>437</v>
       </c>
       <c r="B15" s="15" t="s">
-        <v>427</v>
+        <v>430</v>
       </c>
       <c r="C15" s="17"/>
       <c r="D15" s="15" t="s">
-        <v>426</v>
+        <v>429</v>
       </c>
       <c r="E15" s="15" t="s">
-        <v>426</v>
+        <v>429</v>
       </c>
       <c r="F15" s="15" t="s">
-        <v>434</v>
+        <v>437</v>
       </c>
       <c r="G15" s="15" t="s">
-        <v>428</v>
+        <v>431</v>
       </c>
       <c r="H15" s="15" t="s">
-        <v>428</v>
+        <v>431</v>
       </c>
       <c r="I15" s="18"/>
     </row>
     <row r="17" spans="1:3">
       <c r="A17" t="s">
-        <v>437</v>
+        <v>440</v>
       </c>
       <c r="B17" t="s">
-        <v>438</v>
+        <v>441</v>
       </c>
       <c r="C17" t="s">
-        <v>439</v>
+        <v>442</v>
       </c>
     </row>
     <row r="18" spans="1:3">
       <c r="A18" t="s">
-        <v>438</v>
+        <v>441</v>
       </c>
       <c r="B18" t="s">
-        <v>440</v>
+        <v>443</v>
       </c>
       <c r="C18" t="s">
-        <v>441</v>
+        <v>444</v>
       </c>
     </row>
     <row r="19" spans="1:3">
       <c r="A19" t="s">
-        <v>439</v>
+        <v>442</v>
       </c>
       <c r="B19" t="s">
-        <v>441</v>
+        <v>444</v>
       </c>
       <c r="C19" t="s">
-        <v>442</v>
+        <v>445</v>
       </c>
     </row>
     <row r="21" spans="1:3">
       <c r="A21" t="s">
-        <v>440</v>
+        <v>443</v>
       </c>
       <c r="B21" t="s">
-        <v>443</v>
+        <v>446</v>
       </c>
     </row>
     <row r="22" spans="1:3">
       <c r="A22" t="s">
-        <v>441</v>
+        <v>444</v>
       </c>
       <c r="B22" t="s">
-        <v>444</v>
+        <v>447</v>
       </c>
     </row>
     <row r="23" spans="1:3">
       <c r="A23" t="s">
-        <v>442</v>
+        <v>445</v>
       </c>
       <c r="B23" t="s">
-        <v>445</v>
+        <v>448</v>
       </c>
     </row>
     <row r="25" spans="1:3">
       <c r="A25" t="s">
-        <v>446</v>
+        <v>449</v>
       </c>
     </row>
     <row r="26" spans="1:3">
       <c r="A26" t="s">
-        <v>438</v>
+        <v>441</v>
       </c>
       <c r="B26" t="s">
-        <v>447</v>
+        <v>450</v>
       </c>
       <c r="C26" t="s">
-        <v>448</v>
+        <v>451</v>
       </c>
     </row>
     <row r="28" spans="1:3">
       <c r="B28" t="s">
-        <v>449</v>
+        <v>452</v>
       </c>
     </row>
   </sheetData>
@@ -7982,125 +8053,125 @@
   <sheetData>
     <row r="1" spans="1:7">
       <c r="A1" t="s">
-        <v>450</v>
+        <v>453</v>
       </c>
     </row>
     <row r="2" spans="1:7">
       <c r="A2" t="s">
-        <v>451</v>
+        <v>454</v>
       </c>
     </row>
     <row r="3" spans="1:7">
       <c r="A3" t="s">
-        <v>452</v>
+        <v>455</v>
       </c>
     </row>
     <row r="5" ht="14.25" spans="1:7">
       <c r="A5" t="s">
-        <v>453</v>
+        <v>456</v>
       </c>
       <c r="E5" t="s">
-        <v>454</v>
+        <v>457</v>
       </c>
     </row>
     <row r="6" ht="14.25" spans="1:7">
       <c r="A6" s="13" t="s">
-        <v>455</v>
+        <v>458</v>
       </c>
       <c r="B6" s="13" t="s">
-        <v>456</v>
+        <v>459</v>
       </c>
       <c r="C6" s="13" t="s">
-        <v>457</v>
+        <v>460</v>
       </c>
       <c r="E6" s="13" t="s">
-        <v>455</v>
+        <v>458</v>
       </c>
       <c r="F6" s="13" t="s">
-        <v>458</v>
+        <v>461</v>
       </c>
       <c r="G6" s="13" t="s">
-        <v>459</v>
+        <v>462</v>
       </c>
     </row>
     <row r="7" ht="27.75" spans="1:7">
       <c r="A7" s="14" t="s">
-        <v>460</v>
+        <v>463</v>
       </c>
       <c r="B7" s="14" t="s">
-        <v>461</v>
+        <v>464</v>
       </c>
       <c r="C7" s="14" t="s">
-        <v>462</v>
+        <v>465</v>
       </c>
       <c r="E7" s="14" t="s">
-        <v>463</v>
+        <v>466</v>
       </c>
       <c r="F7" s="14" t="s">
-        <v>464</v>
+        <v>467</v>
       </c>
       <c r="G7" s="14" t="s">
-        <v>465</v>
+        <v>468</v>
       </c>
     </row>
     <row r="8" ht="41.25" spans="1:7">
       <c r="A8" s="14" t="s">
-        <v>466</v>
+        <v>469</v>
       </c>
       <c r="B8" s="14" t="s">
-        <v>467</v>
+        <v>470</v>
       </c>
       <c r="C8" s="14" t="s">
-        <v>468</v>
+        <v>471</v>
       </c>
       <c r="E8" s="14" t="s">
-        <v>469</v>
+        <v>472</v>
       </c>
       <c r="F8" s="14" t="s">
-        <v>470</v>
+        <v>473</v>
       </c>
       <c r="G8" s="14" t="s">
-        <v>471</v>
+        <v>474</v>
       </c>
     </row>
     <row r="9" ht="27.75" spans="1:7">
       <c r="A9" s="14" t="s">
-        <v>472</v>
+        <v>475</v>
       </c>
       <c r="B9" s="14" t="s">
-        <v>473</v>
+        <v>476</v>
       </c>
       <c r="C9" s="14" t="s">
-        <v>474</v>
+        <v>477</v>
       </c>
       <c r="E9" s="14" t="s">
-        <v>475</v>
+        <v>478</v>
       </c>
       <c r="F9" s="14" t="s">
-        <v>476</v>
+        <v>479</v>
       </c>
       <c r="G9" s="14" t="s">
-        <v>477</v>
+        <v>480</v>
       </c>
     </row>
     <row r="10" ht="41.25" spans="1:7">
       <c r="A10" s="14" t="s">
-        <v>478</v>
+        <v>481</v>
       </c>
       <c r="B10" s="14" t="s">
-        <v>479</v>
+        <v>482</v>
       </c>
       <c r="C10" s="14" t="s">
-        <v>480</v>
+        <v>483</v>
       </c>
       <c r="E10" s="14" t="s">
-        <v>481</v>
+        <v>484</v>
       </c>
       <c r="F10" s="14" t="s">
-        <v>482</v>
+        <v>485</v>
       </c>
       <c r="G10" s="14" t="s">
-        <v>483</v>
+        <v>486</v>
       </c>
     </row>
     <row r="11" ht="27.75" spans="1:7">
@@ -8108,64 +8179,64 @@
       <c r="B11" s="14"/>
       <c r="C11" s="14"/>
       <c r="E11" s="14" t="s">
-        <v>484</v>
+        <v>487</v>
       </c>
       <c r="F11" s="14" t="s">
-        <v>485</v>
+        <v>488</v>
       </c>
       <c r="G11" s="14" t="s">
-        <v>486</v>
+        <v>489</v>
       </c>
     </row>
     <row r="12" ht="27.75" spans="1:7">
       <c r="E12" s="14" t="s">
-        <v>487</v>
+        <v>490</v>
       </c>
       <c r="F12" s="14" t="s">
-        <v>488</v>
+        <v>491</v>
       </c>
       <c r="G12" s="14" t="s">
-        <v>489</v>
+        <v>492</v>
       </c>
     </row>
     <row r="13" ht="27.75" spans="1:7">
       <c r="A13" s="13" t="s">
-        <v>490</v>
+        <v>493</v>
       </c>
       <c r="B13" s="13" t="s">
-        <v>458</v>
+        <v>461</v>
       </c>
       <c r="C13" s="13" t="s">
-        <v>491</v>
+        <v>494</v>
       </c>
       <c r="E13" t="s">
-        <v>492</v>
+        <v>495</v>
       </c>
       <c r="F13" t="s">
-        <v>493</v>
+        <v>496</v>
       </c>
       <c r="G13" s="14" t="s">
-        <v>494</v>
+        <v>497</v>
       </c>
     </row>
     <row r="14" ht="27.75" spans="1:7">
       <c r="A14" s="14" t="s">
-        <v>495</v>
+        <v>498</v>
       </c>
       <c r="B14" s="14" t="s">
-        <v>496</v>
+        <v>499</v>
       </c>
       <c r="C14" s="14" t="s">
-        <v>497</v>
+        <v>500</v>
       </c>
       <c r="E14" t="s">
-        <v>498</v>
+        <v>501</v>
       </c>
       <c r="F14" t="s">
-        <v>499</v>
+        <v>502</v>
       </c>
       <c r="G14" s="14" t="s">
-        <v>500</v>
+        <v>503</v>
       </c>
     </row>
     <row r="15" ht="27.75" spans="1:7">
@@ -8173,225 +8244,225 @@
         <v>253</v>
       </c>
       <c r="B15" s="14" t="s">
-        <v>501</v>
+        <v>504</v>
       </c>
       <c r="C15" s="14" t="s">
-        <v>502</v>
+        <v>505</v>
       </c>
       <c r="E15" t="s">
-        <v>503</v>
+        <v>506</v>
       </c>
       <c r="F15" t="s">
-        <v>504</v>
+        <v>507</v>
       </c>
       <c r="G15" s="14" t="s">
-        <v>505</v>
+        <v>508</v>
       </c>
     </row>
     <row r="16" ht="27.75" spans="1:7">
       <c r="A16" s="14" t="s">
-        <v>506</v>
+        <v>509</v>
       </c>
       <c r="B16" s="14" t="s">
-        <v>507</v>
+        <v>510</v>
       </c>
       <c r="C16" s="14" t="s">
-        <v>508</v>
+        <v>511</v>
       </c>
     </row>
     <row r="17" ht="27.75" spans="1:7">
       <c r="A17" s="14" t="s">
-        <v>509</v>
+        <v>512</v>
       </c>
       <c r="B17" s="14" t="s">
-        <v>510</v>
+        <v>513</v>
       </c>
       <c r="C17" s="14" t="s">
-        <v>511</v>
+        <v>514</v>
       </c>
       <c r="E17" s="13" t="s">
-        <v>490</v>
+        <v>493</v>
       </c>
       <c r="F17" s="13" t="s">
-        <v>458</v>
+        <v>461</v>
       </c>
       <c r="G17" s="13" t="s">
-        <v>491</v>
+        <v>494</v>
       </c>
     </row>
     <row r="18" ht="27.75" spans="1:7">
       <c r="A18" s="14" t="s">
-        <v>512</v>
+        <v>515</v>
       </c>
       <c r="B18" s="14" t="s">
-        <v>510</v>
+        <v>513</v>
       </c>
       <c r="C18" s="14" t="s">
-        <v>513</v>
+        <v>516</v>
       </c>
       <c r="E18" s="14" t="s">
         <v>158</v>
       </c>
       <c r="F18" s="14" t="s">
-        <v>514</v>
+        <v>517</v>
       </c>
       <c r="G18" s="14" t="s">
-        <v>515</v>
+        <v>518</v>
       </c>
     </row>
     <row r="19" ht="27.75" spans="1:7">
       <c r="A19" t="s">
-        <v>516</v>
+        <v>519</v>
       </c>
       <c r="B19" t="s">
-        <v>517</v>
+        <v>520</v>
       </c>
       <c r="C19" s="14" t="s">
-        <v>518</v>
+        <v>521</v>
       </c>
       <c r="E19" s="14" t="s">
         <v>265</v>
       </c>
       <c r="F19" s="14" t="s">
-        <v>519</v>
+        <v>522</v>
       </c>
       <c r="G19" s="14" t="s">
-        <v>520</v>
+        <v>523</v>
       </c>
     </row>
     <row r="20" ht="27.75" spans="1:7">
       <c r="E20" s="14" t="s">
-        <v>495</v>
+        <v>498</v>
       </c>
       <c r="F20" s="14" t="s">
-        <v>521</v>
+        <v>524</v>
       </c>
       <c r="G20" s="14" t="s">
-        <v>522</v>
+        <v>525</v>
       </c>
     </row>
     <row r="21" ht="27.75" spans="1:7">
       <c r="E21" t="s">
-        <v>523</v>
+        <v>526</v>
       </c>
       <c r="F21" s="14" t="s">
-        <v>464</v>
+        <v>467</v>
       </c>
       <c r="G21" s="14" t="s">
-        <v>465</v>
+        <v>468</v>
       </c>
     </row>
     <row r="22" ht="27" spans="1:7">
       <c r="E22" t="s">
-        <v>524</v>
+        <v>527</v>
       </c>
       <c r="F22" t="s">
-        <v>525</v>
+        <v>528</v>
       </c>
       <c r="G22" s="6" t="s">
-        <v>526</v>
+        <v>529</v>
       </c>
     </row>
     <row r="23" ht="14.25" spans="1:7">
       <c r="E23" t="s">
-        <v>527</v>
+        <v>530</v>
       </c>
       <c r="F23" t="s">
-        <v>528</v>
+        <v>531</v>
       </c>
       <c r="G23" t="s">
-        <v>529</v>
+        <v>532</v>
       </c>
     </row>
     <row r="24" ht="27.75" spans="1:7">
       <c r="E24" s="14" t="s">
-        <v>495</v>
+        <v>498</v>
       </c>
       <c r="F24" s="14" t="s">
-        <v>530</v>
+        <v>533</v>
       </c>
       <c r="G24" s="14" t="s">
-        <v>522</v>
+        <v>525</v>
       </c>
     </row>
     <row r="26" spans="1:7">
       <c r="A26" t="s">
-        <v>531</v>
+        <v>534</v>
       </c>
       <c r="E26" t="s">
-        <v>532</v>
+        <v>535</v>
       </c>
     </row>
     <row r="27" ht="14.25"/>
     <row r="28" ht="14.25" spans="1:7">
       <c r="A28" s="13" t="s">
-        <v>455</v>
+        <v>458</v>
       </c>
       <c r="B28" s="13" t="s">
+        <v>461</v>
+      </c>
+      <c r="C28" s="13" t="s">
+        <v>462</v>
+      </c>
+      <c r="E28" s="13" t="s">
         <v>458</v>
       </c>
-      <c r="C28" s="13" t="s">
-        <v>459</v>
-      </c>
-      <c r="E28" s="13" t="s">
-        <v>455</v>
-      </c>
       <c r="F28" s="13" t="s">
-        <v>458</v>
+        <v>461</v>
       </c>
       <c r="G28" s="13" t="s">
-        <v>459</v>
+        <v>462</v>
       </c>
     </row>
     <row r="29" ht="54.75" spans="1:7">
       <c r="A29" s="14" t="s">
-        <v>533</v>
+        <v>536</v>
       </c>
       <c r="B29" s="14" t="s">
-        <v>534</v>
+        <v>537</v>
       </c>
       <c r="C29" s="14" t="s">
-        <v>535</v>
+        <v>538</v>
       </c>
       <c r="E29" s="14" t="s">
-        <v>536</v>
+        <v>539</v>
       </c>
       <c r="F29" t="s">
-        <v>537</v>
+        <v>540</v>
       </c>
       <c r="G29" s="14" t="s">
-        <v>538</v>
+        <v>541</v>
       </c>
     </row>
     <row r="30" ht="27.75" spans="1:7">
       <c r="A30" s="14" t="s">
-        <v>539</v>
+        <v>542</v>
       </c>
       <c r="B30" s="14" t="s">
-        <v>534</v>
+        <v>537</v>
       </c>
       <c r="C30" s="14" t="s">
-        <v>535</v>
+        <v>538</v>
       </c>
       <c r="E30" s="14" t="s">
-        <v>540</v>
+        <v>543</v>
       </c>
       <c r="F30" s="14" t="s">
-        <v>541</v>
+        <v>544</v>
       </c>
       <c r="G30" s="14" t="s">
-        <v>542</v>
+        <v>545</v>
       </c>
     </row>
     <row r="31" ht="27.75" spans="1:7">
       <c r="A31" s="14" t="s">
-        <v>543</v>
+        <v>546</v>
       </c>
       <c r="B31" s="14" t="s">
-        <v>544</v>
+        <v>547</v>
       </c>
       <c r="C31" s="14" t="s">
-        <v>545</v>
+        <v>548</v>
       </c>
       <c r="E31" s="14"/>
       <c r="F31" s="14"/>
@@ -8399,173 +8470,173 @@
     </row>
     <row r="32" ht="27.75" spans="1:7">
       <c r="A32" s="14" t="s">
-        <v>546</v>
+        <v>549</v>
       </c>
       <c r="B32" s="14" t="s">
-        <v>547</v>
+        <v>550</v>
       </c>
       <c r="C32" s="14" t="s">
-        <v>548</v>
+        <v>551</v>
       </c>
       <c r="E32" s="13" t="s">
-        <v>490</v>
+        <v>493</v>
       </c>
       <c r="F32" s="13" t="s">
-        <v>458</v>
+        <v>461</v>
       </c>
       <c r="G32" s="13" t="s">
-        <v>491</v>
+        <v>494</v>
       </c>
     </row>
     <row r="33" ht="27.75" spans="1:7">
       <c r="A33" s="14" t="s">
-        <v>549</v>
+        <v>552</v>
       </c>
       <c r="B33" s="14" t="s">
-        <v>550</v>
+        <v>553</v>
       </c>
       <c r="C33" s="14" t="s">
-        <v>551</v>
+        <v>554</v>
       </c>
       <c r="E33" s="14" t="s">
-        <v>552</v>
+        <v>555</v>
       </c>
       <c r="F33" s="14" t="s">
-        <v>553</v>
+        <v>556</v>
       </c>
       <c r="G33" s="14" t="s">
-        <v>554</v>
+        <v>557</v>
       </c>
     </row>
     <row r="34" ht="27.75" spans="1:7">
       <c r="A34" t="s">
-        <v>555</v>
+        <v>558</v>
       </c>
       <c r="B34" t="s">
-        <v>556</v>
+        <v>559</v>
       </c>
       <c r="C34" s="14" t="s">
-        <v>557</v>
+        <v>560</v>
       </c>
       <c r="E34" s="14" t="s">
-        <v>558</v>
+        <v>561</v>
       </c>
       <c r="F34" s="14" t="s">
-        <v>559</v>
+        <v>562</v>
       </c>
       <c r="G34" s="14" t="s">
-        <v>560</v>
+        <v>563</v>
       </c>
     </row>
     <row r="35" ht="27.75" spans="1:7">
       <c r="A35" t="s">
-        <v>561</v>
+        <v>564</v>
       </c>
       <c r="B35" t="s">
-        <v>562</v>
+        <v>565</v>
       </c>
       <c r="C35" s="6" t="s">
-        <v>563</v>
+        <v>566</v>
       </c>
       <c r="E35" s="14" t="s">
-        <v>564</v>
+        <v>567</v>
       </c>
       <c r="F35" s="14" t="s">
-        <v>565</v>
+        <v>568</v>
       </c>
       <c r="G35" s="14" t="s">
-        <v>566</v>
+        <v>569</v>
       </c>
     </row>
     <row r="36" ht="27.75" spans="1:7">
       <c r="E36" s="14" t="s">
-        <v>495</v>
+        <v>498</v>
       </c>
       <c r="F36" s="14" t="s">
-        <v>567</v>
+        <v>570</v>
       </c>
       <c r="G36" s="14" t="s">
-        <v>568</v>
+        <v>571</v>
       </c>
     </row>
     <row r="37" ht="27.75" spans="1:7">
       <c r="A37" s="13" t="s">
-        <v>490</v>
+        <v>493</v>
       </c>
       <c r="B37" s="13" t="s">
-        <v>458</v>
+        <v>461</v>
       </c>
       <c r="C37" s="13" t="s">
-        <v>491</v>
+        <v>494</v>
       </c>
       <c r="E37" s="14" t="s">
-        <v>569</v>
+        <v>572</v>
       </c>
       <c r="F37" s="14" t="s">
-        <v>570</v>
+        <v>573</v>
       </c>
       <c r="G37" s="14" t="s">
-        <v>571</v>
+        <v>574</v>
       </c>
     </row>
     <row r="38" ht="27.75" spans="1:7">
       <c r="A38" s="14" t="s">
-        <v>572</v>
+        <v>575</v>
       </c>
       <c r="B38" s="14" t="s">
-        <v>573</v>
+        <v>576</v>
       </c>
       <c r="C38" s="14" t="s">
-        <v>574</v>
+        <v>577</v>
       </c>
       <c r="E38" t="s">
-        <v>575</v>
+        <v>578</v>
       </c>
       <c r="F38" s="6" t="s">
-        <v>576</v>
+        <v>579</v>
       </c>
       <c r="G38" s="6" t="s">
-        <v>577</v>
+        <v>580</v>
       </c>
     </row>
     <row r="39" ht="27.75" spans="1:7">
       <c r="A39" s="14" t="s">
-        <v>578</v>
+        <v>581</v>
       </c>
       <c r="B39" s="14" t="s">
-        <v>579</v>
+        <v>582</v>
       </c>
       <c r="C39" s="14" t="s">
-        <v>580</v>
+        <v>583</v>
       </c>
       <c r="E39" t="s">
-        <v>581</v>
+        <v>584</v>
       </c>
       <c r="F39" t="s">
-        <v>582</v>
+        <v>585</v>
       </c>
       <c r="G39" t="s">
-        <v>583</v>
+        <v>586</v>
       </c>
     </row>
     <row r="40" ht="54.75" spans="1:7">
       <c r="A40" s="14" t="s">
-        <v>584</v>
+        <v>587</v>
       </c>
       <c r="B40" s="14" t="s">
-        <v>585</v>
+        <v>588</v>
       </c>
       <c r="C40" s="14" t="s">
-        <v>586</v>
+        <v>589</v>
       </c>
       <c r="E40" t="s">
-        <v>587</v>
+        <v>590</v>
       </c>
       <c r="F40" s="6" t="s">
-        <v>588</v>
+        <v>591</v>
       </c>
       <c r="G40" s="6" t="s">
-        <v>589</v>
+        <v>592</v>
       </c>
     </row>
     <row r="41" ht="54.75" spans="1:7">
@@ -8573,98 +8644,98 @@
         <v>112</v>
       </c>
       <c r="B41" s="14" t="s">
-        <v>590</v>
+        <v>593</v>
       </c>
       <c r="C41" s="14" t="s">
-        <v>591</v>
+        <v>594</v>
       </c>
     </row>
     <row r="42" ht="27.75" spans="1:7">
       <c r="A42" s="14" t="s">
-        <v>495</v>
+        <v>498</v>
       </c>
       <c r="B42" s="14" t="s">
-        <v>592</v>
+        <v>595</v>
       </c>
       <c r="C42" s="14" t="s">
-        <v>586</v>
+        <v>589</v>
       </c>
     </row>
     <row r="43" ht="27.75" spans="1:7">
       <c r="A43" t="s">
-        <v>593</v>
+        <v>596</v>
       </c>
       <c r="B43" t="s">
-        <v>594</v>
+        <v>597</v>
       </c>
       <c r="C43" s="14" t="s">
-        <v>595</v>
+        <v>598</v>
       </c>
     </row>
     <row r="46" spans="1:7">
       <c r="A46" t="s">
-        <v>596</v>
+        <v>599</v>
       </c>
       <c r="B46" t="s">
-        <v>597</v>
+        <v>600</v>
       </c>
       <c r="C46" t="s">
-        <v>598</v>
+        <v>601</v>
       </c>
     </row>
     <row r="47" spans="1:7">
       <c r="A47" t="s">
-        <v>599</v>
+        <v>602</v>
       </c>
       <c r="B47" t="s">
-        <v>600</v>
+        <v>603</v>
       </c>
       <c r="C47" t="s">
-        <v>601</v>
+        <v>604</v>
       </c>
     </row>
     <row r="48" spans="1:7">
       <c r="A48" t="s">
-        <v>602</v>
+        <v>605</v>
       </c>
       <c r="B48" t="s">
-        <v>603</v>
+        <v>606</v>
       </c>
       <c r="C48" t="s">
-        <v>604</v>
+        <v>607</v>
       </c>
     </row>
     <row r="49" spans="1:3">
       <c r="A49" t="s">
-        <v>605</v>
+        <v>608</v>
       </c>
       <c r="B49" t="s">
-        <v>606</v>
+        <v>609</v>
       </c>
       <c r="C49" t="s">
-        <v>607</v>
+        <v>610</v>
       </c>
     </row>
     <row r="50" spans="1:3">
       <c r="A50" t="s">
-        <v>608</v>
+        <v>611</v>
       </c>
       <c r="B50" t="s">
-        <v>609</v>
+        <v>612</v>
       </c>
       <c r="C50" t="s">
-        <v>610</v>
+        <v>613</v>
       </c>
     </row>
     <row r="51" spans="1:3">
       <c r="A51" t="s">
-        <v>611</v>
+        <v>614</v>
       </c>
       <c r="B51" t="s">
-        <v>612</v>
+        <v>615</v>
       </c>
       <c r="C51" t="s">
-        <v>613</v>
+        <v>616</v>
       </c>
     </row>
   </sheetData>
@@ -8685,116 +8756,116 @@
   <sheetData>
     <row r="1" ht="27.75" spans="1:6">
       <c r="A1" s="7" t="s">
-        <v>614</v>
+        <v>617</v>
       </c>
       <c r="B1" s="7" t="s">
-        <v>615</v>
+        <v>618</v>
       </c>
       <c r="C1" s="7" t="s">
-        <v>616</v>
+        <v>619</v>
       </c>
       <c r="D1" s="7" t="s">
-        <v>617</v>
+        <v>620</v>
       </c>
       <c r="E1" s="7" t="s">
-        <v>618</v>
+        <v>621</v>
       </c>
       <c r="F1" s="7" t="s">
-        <v>619</v>
+        <v>622</v>
       </c>
     </row>
     <row r="2" ht="14.25" spans="1:6">
       <c r="A2" s="7" t="s">
-        <v>620</v>
+        <v>623</v>
       </c>
       <c r="B2" s="8" t="s">
-        <v>621</v>
+        <v>624</v>
       </c>
       <c r="C2" s="9" t="s">
-        <v>622</v>
+        <v>625</v>
       </c>
       <c r="D2" s="9" t="s">
-        <v>623</v>
+        <v>626</v>
       </c>
       <c r="E2" s="9" t="s">
-        <v>624</v>
+        <v>627</v>
       </c>
       <c r="F2" s="8" t="s">
-        <v>625</v>
+        <v>628</v>
       </c>
     </row>
     <row r="3" ht="14.25" spans="1:6">
       <c r="A3" s="7"/>
       <c r="B3" s="10" t="s">
-        <v>626</v>
+        <v>629</v>
       </c>
       <c r="C3" s="9"/>
       <c r="D3" s="9"/>
       <c r="E3" s="9"/>
       <c r="F3" s="10" t="s">
-        <v>627</v>
+        <v>630</v>
       </c>
     </row>
     <row r="4" ht="14.25" spans="1:6">
       <c r="A4" s="7"/>
       <c r="B4" s="11" t="s">
-        <v>628</v>
+        <v>631</v>
       </c>
       <c r="C4" s="9"/>
       <c r="D4" s="9"/>
       <c r="E4" s="9"/>
       <c r="F4" s="11" t="s">
-        <v>629</v>
+        <v>632</v>
       </c>
     </row>
     <row r="5" ht="27.75" spans="1:6">
       <c r="A5" s="7" t="s">
-        <v>630</v>
+        <v>633</v>
       </c>
       <c r="B5" s="8" t="s">
-        <v>631</v>
+        <v>634</v>
       </c>
       <c r="C5" s="9" t="s">
-        <v>632</v>
+        <v>635</v>
       </c>
       <c r="D5" s="9" t="s">
-        <v>623</v>
+        <v>626</v>
       </c>
       <c r="E5" s="9" t="s">
-        <v>624</v>
+        <v>627</v>
       </c>
       <c r="F5" s="8" t="s">
-        <v>633</v>
+        <v>636</v>
       </c>
     </row>
     <row r="6" ht="14.25" spans="1:6">
       <c r="A6" s="7"/>
       <c r="B6" s="10" t="s">
-        <v>634</v>
+        <v>637</v>
       </c>
       <c r="C6" s="9"/>
       <c r="D6" s="9"/>
       <c r="E6" s="9"/>
       <c r="F6" s="10" t="s">
-        <v>635</v>
+        <v>638</v>
       </c>
     </row>
     <row r="7" ht="14.25" spans="1:6">
       <c r="A7" s="7"/>
       <c r="B7" s="10" t="s">
-        <v>636</v>
+        <v>639</v>
       </c>
       <c r="C7" s="9"/>
       <c r="D7" s="9"/>
       <c r="E7" s="9"/>
       <c r="F7" s="10" t="s">
-        <v>637</v>
+        <v>640</v>
       </c>
     </row>
     <row r="8" ht="14.25" spans="1:6">
       <c r="A8" s="7"/>
       <c r="B8" s="11" t="s">
-        <v>638</v>
+        <v>641</v>
       </c>
       <c r="C8" s="9"/>
       <c r="D8" s="9"/>
@@ -8803,52 +8874,52 @@
     </row>
     <row r="9" ht="14.25" spans="1:6">
       <c r="A9" s="7" t="s">
-        <v>639</v>
+        <v>642</v>
       </c>
       <c r="B9" s="8" t="s">
-        <v>640</v>
+        <v>643</v>
       </c>
       <c r="C9" s="9" t="s">
-        <v>641</v>
+        <v>644</v>
       </c>
       <c r="D9" s="9" t="s">
-        <v>642</v>
+        <v>645</v>
       </c>
       <c r="E9" s="9" t="s">
-        <v>643</v>
+        <v>646</v>
       </c>
       <c r="F9" s="8" t="s">
-        <v>644</v>
+        <v>647</v>
       </c>
     </row>
     <row r="10" ht="14.25" spans="1:6">
       <c r="A10" s="7"/>
       <c r="B10" s="10" t="s">
-        <v>645</v>
+        <v>648</v>
       </c>
       <c r="C10" s="9"/>
       <c r="D10" s="9"/>
       <c r="E10" s="9"/>
       <c r="F10" s="10" t="s">
-        <v>646</v>
+        <v>649</v>
       </c>
     </row>
     <row r="11" ht="14.25" spans="1:6">
       <c r="A11" s="7"/>
       <c r="B11" s="10" t="s">
-        <v>647</v>
+        <v>650</v>
       </c>
       <c r="C11" s="9"/>
       <c r="D11" s="9"/>
       <c r="E11" s="9"/>
       <c r="F11" s="10" t="s">
-        <v>648</v>
+        <v>651</v>
       </c>
     </row>
     <row r="12" ht="14.25" spans="1:6">
       <c r="A12" s="7"/>
       <c r="B12" s="11" t="s">
-        <v>649</v>
+        <v>652</v>
       </c>
       <c r="C12" s="9"/>
       <c r="D12" s="9"/>
@@ -8857,52 +8928,52 @@
     </row>
     <row r="13" ht="27.75" spans="1:6">
       <c r="A13" s="7" t="s">
-        <v>650</v>
+        <v>653</v>
       </c>
       <c r="B13" s="8" t="s">
-        <v>651</v>
+        <v>654</v>
       </c>
       <c r="C13" s="9" t="s">
-        <v>652</v>
+        <v>655</v>
       </c>
       <c r="D13" s="9" t="s">
-        <v>643</v>
+        <v>646</v>
       </c>
       <c r="E13" s="9" t="s">
-        <v>653</v>
+        <v>656</v>
       </c>
       <c r="F13" s="8" t="s">
-        <v>654</v>
+        <v>657</v>
       </c>
     </row>
     <row r="14" ht="14.25" spans="1:6">
       <c r="A14" s="7"/>
       <c r="B14" s="10" t="s">
-        <v>655</v>
+        <v>658</v>
       </c>
       <c r="C14" s="9"/>
       <c r="D14" s="9"/>
       <c r="E14" s="9"/>
       <c r="F14" s="10" t="s">
-        <v>656</v>
+        <v>659</v>
       </c>
     </row>
     <row r="15" ht="14.25" spans="1:6">
       <c r="A15" s="7"/>
       <c r="B15" s="10" t="s">
-        <v>657</v>
+        <v>660</v>
       </c>
       <c r="C15" s="9"/>
       <c r="D15" s="9"/>
       <c r="E15" s="9"/>
       <c r="F15" s="10" t="s">
-        <v>658</v>
+        <v>661</v>
       </c>
     </row>
     <row r="16" ht="14.25" spans="1:6">
       <c r="A16" s="7"/>
       <c r="B16" s="11" t="s">
-        <v>659</v>
+        <v>662</v>
       </c>
       <c r="C16" s="9"/>
       <c r="D16" s="9"/>
@@ -8911,52 +8982,52 @@
     </row>
     <row r="17" ht="14.25" spans="1:6">
       <c r="A17" s="7" t="s">
-        <v>660</v>
+        <v>663</v>
       </c>
       <c r="B17" s="8" t="s">
-        <v>661</v>
+        <v>664</v>
       </c>
       <c r="C17" s="9" t="s">
-        <v>662</v>
+        <v>665</v>
       </c>
       <c r="D17" s="9" t="s">
-        <v>663</v>
+        <v>666</v>
       </c>
       <c r="E17" s="9" t="s">
-        <v>642</v>
+        <v>645</v>
       </c>
       <c r="F17" s="8" t="s">
-        <v>664</v>
+        <v>667</v>
       </c>
     </row>
     <row r="18" ht="14.25" spans="1:6">
       <c r="A18" s="7"/>
       <c r="B18" s="10" t="s">
-        <v>665</v>
+        <v>668</v>
       </c>
       <c r="C18" s="9"/>
       <c r="D18" s="9"/>
       <c r="E18" s="9"/>
       <c r="F18" s="10" t="s">
-        <v>666</v>
+        <v>669</v>
       </c>
     </row>
     <row r="19" ht="14.25" spans="1:6">
       <c r="A19" s="7"/>
       <c r="B19" s="10" t="s">
-        <v>667</v>
+        <v>670</v>
       </c>
       <c r="C19" s="9"/>
       <c r="D19" s="9"/>
       <c r="E19" s="9"/>
       <c r="F19" s="10" t="s">
-        <v>668</v>
+        <v>671</v>
       </c>
     </row>
     <row r="20" ht="14.25" spans="1:6">
       <c r="A20" s="7"/>
       <c r="B20" s="11" t="s">
-        <v>669</v>
+        <v>672</v>
       </c>
       <c r="C20" s="9"/>
       <c r="D20" s="9"/>
@@ -8965,52 +9036,52 @@
     </row>
     <row r="21" ht="27.75" spans="1:6">
       <c r="A21" s="7" t="s">
-        <v>670</v>
+        <v>673</v>
       </c>
       <c r="B21" s="8" t="s">
-        <v>671</v>
+        <v>674</v>
       </c>
       <c r="C21" s="9" t="s">
-        <v>672</v>
+        <v>675</v>
       </c>
       <c r="D21" s="9" t="s">
-        <v>623</v>
+        <v>626</v>
       </c>
       <c r="E21" s="9" t="s">
-        <v>663</v>
+        <v>666</v>
       </c>
       <c r="F21" s="8" t="s">
-        <v>673</v>
+        <v>676</v>
       </c>
     </row>
     <row r="22" ht="14.25" spans="1:6">
       <c r="A22" s="7"/>
       <c r="B22" s="10" t="s">
-        <v>674</v>
+        <v>677</v>
       </c>
       <c r="C22" s="9"/>
       <c r="D22" s="9"/>
       <c r="E22" s="9"/>
       <c r="F22" s="10" t="s">
-        <v>675</v>
+        <v>678</v>
       </c>
     </row>
     <row r="23" ht="14.25" spans="1:6">
       <c r="A23" s="7"/>
       <c r="B23" s="10" t="s">
-        <v>676</v>
+        <v>679</v>
       </c>
       <c r="C23" s="9"/>
       <c r="D23" s="9"/>
       <c r="E23" s="9"/>
       <c r="F23" s="10" t="s">
-        <v>677</v>
+        <v>680</v>
       </c>
     </row>
     <row r="24" ht="14.25" spans="1:6">
       <c r="A24" s="7"/>
       <c r="B24" s="11" t="s">
-        <v>678</v>
+        <v>681</v>
       </c>
       <c r="C24" s="9"/>
       <c r="D24" s="9"/>
@@ -9062,7 +9133,7 @@
     </row>
     <row r="2" spans="1:2">
       <c r="A2" t="s">
-        <v>450</v>
+        <v>453</v>
       </c>
     </row>
     <row r="3" spans="1:2">
@@ -9070,7 +9141,7 @@
         <v>1</v>
       </c>
       <c r="B3" t="s">
-        <v>679</v>
+        <v>682</v>
       </c>
     </row>
     <row r="4" spans="1:2">
@@ -9078,7 +9149,7 @@
         <v>2</v>
       </c>
       <c r="B4" t="s">
-        <v>680</v>
+        <v>683</v>
       </c>
     </row>
     <row r="5" spans="1:2">
@@ -9086,7 +9157,7 @@
         <v>3</v>
       </c>
       <c r="B5" t="s">
-        <v>681</v>
+        <v>684</v>
       </c>
     </row>
     <row r="6" spans="1:2">
@@ -9094,7 +9165,7 @@
         <v>4</v>
       </c>
       <c r="B6" t="s">
-        <v>682</v>
+        <v>685</v>
       </c>
     </row>
     <row r="7" spans="1:2">
@@ -9102,7 +9173,7 @@
         <v>5</v>
       </c>
       <c r="B7" t="s">
-        <v>683</v>
+        <v>686</v>
       </c>
     </row>
     <row r="8" spans="1:2">
@@ -9110,227 +9181,227 @@
         <v>6</v>
       </c>
       <c r="B8" t="s">
-        <v>684</v>
+        <v>687</v>
       </c>
     </row>
     <row r="10" spans="1:2">
       <c r="A10" t="s">
-        <v>685</v>
+        <v>688</v>
       </c>
     </row>
     <row r="11" spans="1:2">
       <c r="A11" t="s">
-        <v>686</v>
+        <v>689</v>
       </c>
     </row>
     <row r="12" spans="1:2">
       <c r="A12" t="s">
-        <v>687</v>
+        <v>690</v>
       </c>
     </row>
     <row r="13" spans="1:2">
       <c r="A13" t="s">
-        <v>688</v>
+        <v>691</v>
       </c>
       <c r="B13" t="s">
-        <v>689</v>
+        <v>692</v>
       </c>
     </row>
     <row r="14" spans="1:2">
       <c r="A14" t="s">
-        <v>690</v>
+        <v>693</v>
       </c>
       <c r="B14" t="s">
-        <v>691</v>
+        <v>694</v>
       </c>
     </row>
     <row r="15" spans="1:2">
       <c r="A15" t="s">
-        <v>692</v>
+        <v>695</v>
       </c>
       <c r="B15" t="s">
-        <v>693</v>
+        <v>696</v>
       </c>
     </row>
     <row r="16" spans="1:2">
       <c r="A16" t="s">
-        <v>694</v>
+        <v>697</v>
       </c>
       <c r="B16" t="s">
-        <v>695</v>
+        <v>698</v>
       </c>
     </row>
     <row r="17" spans="1:2">
       <c r="A17" t="s">
-        <v>696</v>
+        <v>699</v>
       </c>
       <c r="B17" t="s">
-        <v>697</v>
+        <v>700</v>
       </c>
     </row>
     <row r="18" spans="1:2">
       <c r="A18" t="s">
-        <v>698</v>
+        <v>701</v>
       </c>
       <c r="B18" t="s">
-        <v>699</v>
+        <v>702</v>
       </c>
     </row>
     <row r="19" spans="1:2">
       <c r="A19" t="s">
-        <v>700</v>
+        <v>703</v>
       </c>
     </row>
     <row r="20" spans="1:2">
       <c r="A20" t="s">
-        <v>701</v>
+        <v>704</v>
       </c>
       <c r="B20" t="s">
-        <v>702</v>
+        <v>705</v>
       </c>
     </row>
     <row r="21" spans="1:2">
       <c r="A21" t="s">
-        <v>703</v>
+        <v>706</v>
       </c>
       <c r="B21" t="s">
-        <v>704</v>
+        <v>707</v>
       </c>
     </row>
     <row r="22" spans="1:2">
       <c r="A22" t="s">
-        <v>705</v>
+        <v>708</v>
       </c>
       <c r="B22" t="s">
-        <v>706</v>
+        <v>709</v>
       </c>
     </row>
     <row r="23" spans="1:2">
       <c r="A23" t="s">
-        <v>707</v>
+        <v>710</v>
       </c>
       <c r="B23" t="s">
-        <v>708</v>
+        <v>711</v>
       </c>
     </row>
     <row r="24" spans="1:2">
       <c r="A24" t="s">
-        <v>709</v>
+        <v>712</v>
       </c>
       <c r="B24" t="s">
-        <v>710</v>
+        <v>713</v>
       </c>
     </row>
     <row r="25" spans="1:2">
       <c r="A25" t="s">
-        <v>711</v>
+        <v>714</v>
       </c>
       <c r="B25" t="s">
-        <v>712</v>
+        <v>715</v>
       </c>
     </row>
     <row r="27" spans="1:2">
       <c r="A27" t="s">
-        <v>713</v>
+        <v>716</v>
       </c>
     </row>
     <row r="28" spans="1:2">
       <c r="A28" t="s">
-        <v>714</v>
+        <v>717</v>
       </c>
       <c r="B28" t="s">
-        <v>715</v>
+        <v>718</v>
       </c>
     </row>
     <row r="29" spans="1:2">
       <c r="A29" t="s">
-        <v>716</v>
+        <v>719</v>
       </c>
       <c r="B29" t="s">
-        <v>717</v>
+        <v>720</v>
       </c>
     </row>
     <row r="30" spans="1:2">
       <c r="B30" t="s">
-        <v>718</v>
+        <v>721</v>
       </c>
     </row>
     <row r="32" spans="1:2">
       <c r="A32" t="s">
-        <v>719</v>
+        <v>722</v>
       </c>
     </row>
     <row r="33" spans="1:7">
       <c r="A33" t="s">
-        <v>714</v>
+        <v>717</v>
       </c>
       <c r="B33" t="s">
-        <v>720</v>
+        <v>723</v>
       </c>
     </row>
     <row r="34" spans="1:7">
       <c r="B34" t="s">
-        <v>721</v>
+        <v>724</v>
       </c>
     </row>
     <row r="35" spans="1:7">
       <c r="B35" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
     </row>
     <row r="36" spans="1:7">
       <c r="B36" t="s">
-        <v>723</v>
+        <v>726</v>
       </c>
     </row>
     <row r="37" spans="1:7">
       <c r="B37" t="s">
-        <v>724</v>
+        <v>727</v>
       </c>
     </row>
     <row r="39" spans="1:7">
       <c r="A39" t="s">
-        <v>725</v>
+        <v>728</v>
       </c>
     </row>
     <row r="40" spans="1:7">
       <c r="A40" t="s">
-        <v>726</v>
+        <v>729</v>
       </c>
       <c r="B40" t="s">
-        <v>727</v>
+        <v>730</v>
       </c>
       <c r="C40" t="s">
         <v>21</v>
       </c>
       <c r="D40" t="s">
-        <v>728</v>
+        <v>731</v>
       </c>
       <c r="E40" t="s">
-        <v>729</v>
+        <v>732</v>
       </c>
       <c r="F40" t="s">
-        <v>730</v>
+        <v>733</v>
       </c>
       <c r="G40" t="s">
-        <v>731</v>
+        <v>734</v>
       </c>
     </row>
     <row r="41" spans="1:7">
       <c r="A41" t="s">
-        <v>732</v>
+        <v>735</v>
       </c>
       <c r="B41" t="s">
-        <v>733</v>
+        <v>736</v>
       </c>
       <c r="C41" t="s">
-        <v>734</v>
+        <v>737</v>
       </c>
       <c r="D41" t="s">
-        <v>735</v>
+        <v>738</v>
       </c>
       <c r="E41" t="s">
-        <v>736</v>
+        <v>739</v>
       </c>
       <c r="F41">
         <v>40</v>
@@ -9341,19 +9412,19 @@
     </row>
     <row r="42" spans="1:7">
       <c r="A42" t="s">
-        <v>737</v>
+        <v>740</v>
       </c>
       <c r="B42" t="s">
-        <v>738</v>
+        <v>741</v>
       </c>
       <c r="C42" t="s">
-        <v>739</v>
+        <v>742</v>
       </c>
       <c r="D42" t="s">
-        <v>740</v>
+        <v>743</v>
       </c>
       <c r="E42" t="s">
-        <v>741</v>
+        <v>744</v>
       </c>
       <c r="F42">
         <v>20</v>
@@ -9364,19 +9435,19 @@
     </row>
     <row r="43" spans="1:7">
       <c r="A43" t="s">
-        <v>742</v>
+        <v>745</v>
       </c>
       <c r="B43" t="s">
-        <v>743</v>
+        <v>746</v>
       </c>
       <c r="C43" t="s">
-        <v>744</v>
+        <v>747</v>
       </c>
       <c r="D43" t="s">
-        <v>745</v>
+        <v>748</v>
       </c>
       <c r="E43" t="s">
-        <v>746</v>
+        <v>749</v>
       </c>
       <c r="F43">
         <v>10</v>
@@ -9387,94 +9458,94 @@
     </row>
     <row r="46" spans="1:7">
       <c r="A46" s="6" t="s">
-        <v>747</v>
+        <v>750</v>
       </c>
       <c r="B46" t="s">
-        <v>748</v>
+        <v>751</v>
       </c>
       <c r="C46" t="s">
-        <v>749</v>
+        <v>752</v>
       </c>
       <c r="D46" t="s">
-        <v>750</v>
+        <v>753</v>
       </c>
       <c r="E46" t="s">
-        <v>751</v>
+        <v>754</v>
       </c>
       <c r="F46" t="s">
-        <v>752</v>
+        <v>755</v>
       </c>
       <c r="G46" t="s">
-        <v>753</v>
+        <v>756</v>
       </c>
     </row>
     <row r="47" spans="1:7">
       <c r="A47" t="s">
-        <v>754</v>
+        <v>757</v>
       </c>
       <c r="B47" t="s">
-        <v>755</v>
+        <v>758</v>
       </c>
       <c r="C47" t="s">
-        <v>756</v>
+        <v>759</v>
       </c>
       <c r="D47" t="s">
-        <v>564</v>
+        <v>567</v>
       </c>
       <c r="E47" t="s">
-        <v>757</v>
+        <v>760</v>
       </c>
       <c r="F47" t="s">
-        <v>758</v>
+        <v>761</v>
       </c>
       <c r="G47" t="s">
-        <v>759</v>
+        <v>762</v>
       </c>
     </row>
     <row r="48" spans="1:7">
       <c r="A48" t="s">
-        <v>760</v>
+        <v>763</v>
       </c>
       <c r="B48" t="s">
-        <v>761</v>
+        <v>764</v>
       </c>
       <c r="C48" t="s">
-        <v>762</v>
+        <v>765</v>
       </c>
       <c r="D48" t="s">
-        <v>763</v>
+        <v>766</v>
       </c>
       <c r="E48" t="s">
-        <v>764</v>
+        <v>767</v>
       </c>
       <c r="F48" t="s">
-        <v>765</v>
+        <v>768</v>
       </c>
       <c r="G48" t="s">
-        <v>766</v>
+        <v>769</v>
       </c>
     </row>
     <row r="49" spans="1:7">
       <c r="A49" t="s">
-        <v>767</v>
+        <v>770</v>
       </c>
       <c r="B49" t="s">
-        <v>768</v>
+        <v>771</v>
       </c>
       <c r="C49" t="s">
-        <v>769</v>
+        <v>772</v>
       </c>
       <c r="D49" t="s">
-        <v>770</v>
+        <v>773</v>
       </c>
       <c r="E49" t="s">
-        <v>771</v>
+        <v>774</v>
       </c>
       <c r="F49" t="s">
-        <v>772</v>
+        <v>775</v>
       </c>
       <c r="G49" t="s">
-        <v>773</v>
+        <v>776</v>
       </c>
     </row>
   </sheetData>
@@ -9495,12 +9566,12 @@
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" t="s">
-        <v>495</v>
+        <v>498</v>
       </c>
     </row>
     <row r="2" spans="1:2">
       <c r="A2" t="s">
-        <v>450</v>
+        <v>453</v>
       </c>
     </row>
     <row r="3" spans="1:2">
@@ -9508,7 +9579,7 @@
         <v>1</v>
       </c>
       <c r="B3" t="s">
-        <v>774</v>
+        <v>777</v>
       </c>
     </row>
     <row r="4" spans="1:2">
@@ -9516,7 +9587,7 @@
         <v>2</v>
       </c>
       <c r="B4" t="s">
-        <v>775</v>
+        <v>778</v>
       </c>
     </row>
     <row r="5" spans="1:2">
@@ -9524,7 +9595,7 @@
         <v>3</v>
       </c>
       <c r="B5" t="s">
-        <v>776</v>
+        <v>779</v>
       </c>
     </row>
     <row r="6" spans="1:2">
@@ -9533,15 +9604,15 @@
     </row>
     <row r="7" spans="1:2">
       <c r="A7" s="2" t="s">
-        <v>777</v>
+        <v>780</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>778</v>
+        <v>781</v>
       </c>
     </row>
     <row r="8" spans="1:2">
       <c r="A8" s="3" t="s">
-        <v>779</v>
+        <v>782</v>
       </c>
       <c r="B8" s="2">
         <v>30</v>
@@ -9549,7 +9620,7 @@
     </row>
     <row r="9" spans="1:2">
       <c r="A9" s="3" t="s">
-        <v>780</v>
+        <v>783</v>
       </c>
       <c r="B9" s="2">
         <v>60</v>
@@ -9557,7 +9628,7 @@
     </row>
     <row r="10" spans="1:2">
       <c r="A10" s="3" t="s">
-        <v>781</v>
+        <v>784</v>
       </c>
       <c r="B10" s="2">
         <v>100</v>
@@ -9565,7 +9636,7 @@
     </row>
     <row r="11" spans="1:2">
       <c r="A11" s="2" t="s">
-        <v>782</v>
+        <v>785</v>
       </c>
       <c r="B11" s="2">
         <v>200</v>
@@ -9573,7 +9644,7 @@
     </row>
     <row r="16" spans="1:2">
       <c r="A16" t="s">
-        <v>783</v>
+        <v>786</v>
       </c>
     </row>
     <row r="18" spans="1:3">
@@ -9581,207 +9652,207 @@
         <v>68</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>784</v>
+        <v>787</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>785</v>
+        <v>788</v>
       </c>
     </row>
     <row r="19" spans="1:3">
       <c r="A19" s="2" t="s">
-        <v>786</v>
+        <v>789</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>787</v>
+        <v>790</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>788</v>
+        <v>791</v>
       </c>
     </row>
     <row r="20" spans="1:3">
       <c r="A20" s="2" t="s">
-        <v>789</v>
+        <v>792</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>787</v>
+        <v>790</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>788</v>
+        <v>791</v>
       </c>
     </row>
     <row r="21" spans="1:3">
       <c r="A21" s="2" t="s">
+        <v>793</v>
+      </c>
+      <c r="B21" s="2" t="s">
         <v>790</v>
       </c>
-      <c r="B21" s="2" t="s">
-        <v>787</v>
-      </c>
       <c r="C21" s="2" t="s">
-        <v>788</v>
+        <v>791</v>
       </c>
     </row>
     <row r="22" spans="1:3">
       <c r="A22" s="2" t="s">
-        <v>791</v>
+        <v>794</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>792</v>
+        <v>795</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>793</v>
+        <v>796</v>
       </c>
     </row>
     <row r="23" spans="1:3">
       <c r="A23" s="2" t="s">
-        <v>794</v>
+        <v>797</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>795</v>
+        <v>798</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>796</v>
+        <v>799</v>
       </c>
     </row>
     <row r="24" spans="1:3">
       <c r="A24" s="2" t="s">
-        <v>797</v>
+        <v>800</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>798</v>
+        <v>801</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>799</v>
+        <v>802</v>
       </c>
     </row>
     <row r="25" spans="1:3">
       <c r="A25" s="2" t="s">
-        <v>800</v>
+        <v>803</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>801</v>
+        <v>804</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>802</v>
+        <v>805</v>
       </c>
     </row>
     <row r="26" spans="1:3">
       <c r="A26" s="2" t="s">
-        <v>803</v>
+        <v>806</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>804</v>
+        <v>807</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>805</v>
+        <v>808</v>
       </c>
     </row>
     <row r="27" spans="1:3">
       <c r="A27" s="2" t="s">
-        <v>806</v>
+        <v>809</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>807</v>
+        <v>810</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>808</v>
+        <v>811</v>
       </c>
     </row>
     <row r="28" spans="1:3">
       <c r="A28" s="2" t="s">
-        <v>809</v>
+        <v>812</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>810</v>
+        <v>813</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>811</v>
+        <v>814</v>
       </c>
     </row>
     <row r="29" spans="1:3">
       <c r="A29" s="2" t="s">
-        <v>812</v>
+        <v>815</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>813</v>
+        <v>816</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>814</v>
+        <v>817</v>
       </c>
     </row>
     <row r="30" spans="1:3">
       <c r="A30" s="4" t="s">
-        <v>815</v>
+        <v>818</v>
       </c>
       <c r="B30" s="4" t="s">
-        <v>816</v>
+        <v>819</v>
       </c>
       <c r="C30" s="4" t="s">
-        <v>817</v>
+        <v>820</v>
       </c>
     </row>
     <row r="31" spans="1:3">
       <c r="A31" s="2" t="s">
-        <v>818</v>
+        <v>821</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>819</v>
+        <v>822</v>
       </c>
       <c r="C31" s="2" t="s">
-        <v>820</v>
+        <v>823</v>
       </c>
     </row>
     <row r="32" spans="1:3">
       <c r="A32" s="2" t="s">
-        <v>821</v>
+        <v>824</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>822</v>
+        <v>825</v>
       </c>
       <c r="C32" s="2" t="s">
-        <v>823</v>
+        <v>826</v>
       </c>
     </row>
     <row r="34" spans="1:8">
       <c r="A34" s="2" t="s">
-        <v>726</v>
+        <v>729</v>
       </c>
       <c r="B34" s="2" t="s">
-        <v>824</v>
+        <v>827</v>
       </c>
       <c r="C34" s="2" t="s">
-        <v>825</v>
+        <v>828</v>
       </c>
       <c r="D34" s="2" t="s">
-        <v>826</v>
+        <v>829</v>
       </c>
       <c r="E34" s="2" t="s">
-        <v>827</v>
+        <v>830</v>
       </c>
       <c r="F34" s="2" t="s">
-        <v>828</v>
+        <v>831</v>
       </c>
       <c r="G34" s="2" t="s">
-        <v>784</v>
+        <v>787</v>
       </c>
       <c r="H34" s="2" t="s">
-        <v>785</v>
+        <v>788</v>
       </c>
     </row>
     <row r="35" spans="1:8">
       <c r="A35" s="2" t="s">
-        <v>732</v>
+        <v>735</v>
       </c>
       <c r="B35" s="2" t="s">
-        <v>786</v>
+        <v>789</v>
       </c>
       <c r="C35" s="2" t="s">
-        <v>829</v>
+        <v>832</v>
       </c>
       <c r="D35" s="2" t="s">
-        <v>806</v>
+        <v>809</v>
       </c>
       <c r="E35" s="2" t="s">
-        <v>815</v>
+        <v>818</v>
       </c>
       <c r="F35" s="2">
         <v>40</v>
@@ -9795,19 +9866,19 @@
     </row>
     <row r="36" spans="1:8">
       <c r="A36" s="2" t="s">
-        <v>737</v>
+        <v>740</v>
       </c>
       <c r="B36" s="2" t="s">
-        <v>830</v>
+        <v>833</v>
       </c>
       <c r="C36" s="2" t="s">
-        <v>831</v>
+        <v>834</v>
       </c>
       <c r="D36" s="2" t="s">
-        <v>809</v>
+        <v>812</v>
       </c>
       <c r="E36" s="2" t="s">
-        <v>818</v>
+        <v>821</v>
       </c>
       <c r="F36" s="2">
         <v>20</v>
@@ -9821,19 +9892,19 @@
     </row>
     <row r="37" spans="1:8">
       <c r="A37" s="2" t="s">
-        <v>832</v>
+        <v>835</v>
       </c>
       <c r="B37" s="2" t="s">
-        <v>833</v>
+        <v>836</v>
       </c>
       <c r="C37" s="2" t="s">
-        <v>803</v>
+        <v>806</v>
       </c>
       <c r="D37" s="2" t="s">
-        <v>812</v>
+        <v>815</v>
       </c>
       <c r="E37" s="2" t="s">
-        <v>821</v>
+        <v>824</v>
       </c>
       <c r="F37" s="2">
         <v>10</v>

</xml_diff>

<commit_message>
P0 safety snapshot before OpenClaw security hardening
- Created for P0.4A protection.
- Temporary recovery snapshot.
- Captures current EOR state before OpenClaw security hardening.
- Remote branch is not a merge target.
</commit_message>
<xml_diff>
--- a/docs/MVP 0.9 项目管理/01_需求与版本规划/EOR MVP 1.0 目标版本规划 V1.1.xlsx
+++ b/docs/MVP 0.9 项目管理/01_需求与版本规划/EOR MVP 1.0 目标版本规划 V1.1.xlsx
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1168" uniqueCount="837">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1171" uniqueCount="839">
   <si>
     <t>人物属性</t>
   </si>
@@ -1390,6 +1390,12 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Segoe UI"/>
+        <charset val="134"/>
+      </rPr>
       <t xml:space="preserve">P0 </t>
     </r>
     <r>
@@ -3311,6 +3317,15 @@
     <t>百夫长</t>
   </si>
   <si>
+    <t>执政官</t>
+  </si>
+  <si>
+    <t>通过法案多于50%</t>
+  </si>
+  <si>
+    <t>通过法案少于50%</t>
+  </si>
+  <si>
     <t>总督</t>
   </si>
   <si>
@@ -3354,9 +3369,6 @@
   </si>
   <si>
     <t>未参与投标</t>
-  </si>
-  <si>
-    <t>执政官</t>
   </si>
   <si>
     <t>影响力上升</t>
@@ -3679,13 +3691,13 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="10"/>
+      <sz val="9"/>
       <color rgb="FF000000"/>
       <name val="Consolas"/>
       <charset val="134"/>
     </font>
     <font>
-      <sz val="9"/>
+      <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Consolas"/>
       <charset val="134"/>
@@ -4710,7 +4722,7 @@
     </dxf>
   </dxfs>
   <tableStyles count="2" defaultTableStyle="TableStylePreset3_Accent1 1" defaultPivotStyle="PivotStylePreset2_Accent1 1">
-    <tableStyle name="TableStylePreset3_Accent1 1" pivot="0" count="7" xr9:uid="{DCD53CD2-7D63-465F-8282-B831EBB5EED1}">
+    <tableStyle name="TableStylePreset3_Accent1 1" pivot="0" count="7" xr9:uid="{AFB8ACB1-2AB2-4505-8814-194619417611}">
       <tableStyleElement type="wholeTable" dxfId="7"/>
       <tableStyleElement type="headerRow" dxfId="6"/>
       <tableStyleElement type="totalRow" dxfId="5"/>
@@ -4719,7 +4731,7 @@
       <tableStyleElement type="firstRowStripe" dxfId="2"/>
       <tableStyleElement type="firstColumnStripe" dxfId="1"/>
     </tableStyle>
-    <tableStyle name="PivotStylePreset2_Accent1 1" table="0" count="10" xr9:uid="{D209FF72-8775-4799-A746-0B9339E74356}">
+    <tableStyle name="PivotStylePreset2_Accent1 1" table="0" count="10" xr9:uid="{E90F00D1-9AB6-4252-8E1A-BCD6604A2FF4}">
       <tableStyleElement type="headerRow" dxfId="17"/>
       <tableStyleElement type="totalRow" dxfId="16"/>
       <tableStyleElement type="firstRowStripe" dxfId="15"/>
@@ -5419,7 +5431,7 @@
       </c>
       <c r="G5" s="2"/>
     </row>
-    <row r="6" ht="27" spans="1:7">
+    <row r="6" ht="27" hidden="1" spans="1:7">
       <c r="A6" s="2" t="s">
         <v>81</v>
       </c>
@@ -5457,7 +5469,7 @@
       <c r="F7" s="2"/>
       <c r="G7" s="2"/>
     </row>
-    <row r="8" ht="16.5" spans="1:7">
+    <row r="8" ht="16.5" hidden="1" spans="1:7">
       <c r="A8" s="2" t="s">
         <v>89</v>
       </c>
@@ -5478,7 +5490,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="9" ht="135" spans="1:7">
+    <row r="9" ht="135" hidden="1" spans="1:7">
       <c r="A9" s="2" t="s">
         <v>92</v>
       </c>
@@ -5499,7 +5511,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="10" ht="27" hidden="1" spans="1:7">
+    <row r="10" ht="27" spans="1:7">
       <c r="A10" s="2" t="s">
         <v>96</v>
       </c>
@@ -5571,7 +5583,7 @@
       <c r="F13" s="2"/>
       <c r="G13" s="2"/>
     </row>
-    <row r="14" ht="27" hidden="1" spans="1:7">
+    <row r="14" ht="27" spans="1:7">
       <c r="A14" s="2" t="s">
         <v>109</v>
       </c>
@@ -5723,7 +5735,7 @@
       </c>
       <c r="G21" s="2"/>
     </row>
-    <row r="22" ht="40.5" hidden="1" spans="1:7">
+    <row r="22" ht="40.5" spans="1:7">
       <c r="A22" s="2" t="s">
         <v>136</v>
       </c>
@@ -5812,7 +5824,7 @@
       <c r="F26" s="2"/>
       <c r="G26" s="2"/>
     </row>
-    <row r="27" ht="43.5" hidden="1" spans="1:7">
+    <row r="27" ht="43.5" spans="1:7">
       <c r="A27" s="2" t="s">
         <v>150</v>
       </c>
@@ -5850,7 +5862,7 @@
       <c r="F28" s="2"/>
       <c r="G28" s="2"/>
     </row>
-    <row r="29" ht="30" hidden="1" spans="1:7">
+    <row r="29" ht="30" spans="1:7">
       <c r="A29" s="2" t="s">
         <v>157</v>
       </c>
@@ -5871,7 +5883,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="30" ht="43.5" hidden="1" spans="1:7">
+    <row r="30" ht="43.5" spans="1:7">
       <c r="A30" s="2" t="s">
         <v>161</v>
       </c>
@@ -5981,7 +5993,7 @@
       </c>
       <c r="G35" s="2"/>
     </row>
-    <row r="36" ht="27" hidden="1" spans="1:7">
+    <row r="36" ht="27" spans="1:7">
       <c r="A36" s="2" t="s">
         <v>179</v>
       </c>
@@ -6337,7 +6349,7 @@
       <c r="F55" s="2"/>
       <c r="G55" s="2"/>
     </row>
-    <row r="56" ht="16.5" hidden="1" spans="1:7">
+    <row r="56" ht="16.5" spans="1:7">
       <c r="A56" s="2" t="s">
         <v>238</v>
       </c>
@@ -6358,7 +6370,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="57" ht="27" hidden="1" spans="1:7">
+    <row r="57" ht="27" spans="1:7">
       <c r="A57" s="2" t="s">
         <v>241</v>
       </c>
@@ -6396,7 +6408,7 @@
       <c r="F58" s="2"/>
       <c r="G58" s="2"/>
     </row>
-    <row r="59" ht="40.5" hidden="1" spans="1:7">
+    <row r="59" ht="40.5" spans="1:7">
       <c r="A59" s="2" t="s">
         <v>248</v>
       </c>
@@ -6417,7 +6429,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="60" ht="27" hidden="1" spans="1:7">
+    <row r="60" ht="27" spans="1:7">
       <c r="A60" s="2" t="s">
         <v>252</v>
       </c>
@@ -6438,7 +6450,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="61" ht="16.5" hidden="1" spans="1:7">
+    <row r="61" ht="16.5" spans="1:7">
       <c r="A61" s="2" t="s">
         <v>255</v>
       </c>
@@ -6493,7 +6505,7 @@
       </c>
       <c r="G63" s="2"/>
     </row>
-    <row r="64" ht="27" hidden="1" spans="1:7">
+    <row r="64" ht="27" spans="1:7">
       <c r="A64" s="2" t="s">
         <v>264</v>
       </c>
@@ -6535,7 +6547,7 @@
       </c>
       <c r="G65" s="2"/>
     </row>
-    <row r="66" ht="43.5" hidden="1" spans="1:7">
+    <row r="66" ht="43.5" spans="1:7">
       <c r="A66" s="2" t="s">
         <v>272</v>
       </c>
@@ -6615,7 +6627,7 @@
       <c r="F69" s="2"/>
       <c r="G69" s="2"/>
     </row>
-    <row r="70" ht="54" hidden="1" spans="1:7">
+    <row r="70" ht="54" spans="1:7">
       <c r="A70" s="2" t="s">
         <v>285</v>
       </c>
@@ -6636,7 +6648,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="71" ht="40.5" hidden="1" spans="1:7">
+    <row r="71" ht="40.5" spans="1:7">
       <c r="A71" s="2" t="s">
         <v>289</v>
       </c>
@@ -6678,7 +6690,7 @@
       </c>
       <c r="G72" s="2"/>
     </row>
-    <row r="73" ht="54" spans="1:7">
+    <row r="73" ht="54" hidden="1" spans="1:7">
       <c r="A73" s="2" t="s">
         <v>297</v>
       </c>
@@ -6927,7 +6939,7 @@
       </c>
       <c r="G87" s="2"/>
     </row>
-    <row r="88" ht="54" hidden="1" spans="1:7">
+    <row r="88" ht="54" spans="1:7">
       <c r="A88" s="2" t="s">
         <v>329</v>
       </c>
@@ -7014,7 +7026,7 @@
       <c r="F92" s="2"/>
       <c r="G92" s="2"/>
     </row>
-    <row r="93" ht="30" hidden="1" spans="1:7">
+    <row r="93" ht="30" spans="1:7">
       <c r="A93" s="2" t="s">
         <v>342</v>
       </c>
@@ -7056,7 +7068,7 @@
       </c>
       <c r="G94" s="2"/>
     </row>
-    <row r="95" ht="57" hidden="1" spans="1:7">
+    <row r="95" ht="57" spans="1:7">
       <c r="A95" s="2" t="s">
         <v>349</v>
       </c>
@@ -7132,7 +7144,7 @@
       <c r="F98" s="2"/>
       <c r="G98" s="2"/>
     </row>
-    <row r="99" customFormat="1" ht="40.5" hidden="1" spans="1:7">
+    <row r="99" customFormat="1" ht="40.5" spans="1:7">
       <c r="A99" s="2" t="s">
         <v>361</v>
       </c>
@@ -7254,7 +7266,7 @@
       </c>
       <c r="G104" s="2"/>
     </row>
-    <row r="105" customFormat="1" ht="40.5" hidden="1" spans="1:7">
+    <row r="105" customFormat="1" ht="40.5" spans="1:7">
       <c r="A105" s="2" t="s">
         <v>383</v>
       </c>
@@ -7309,7 +7321,7 @@
   <autoFilter xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" ref="A3:G105" etc:filterBottomFollowUsedRange="0">
     <filterColumn colId="4">
       <filters>
-        <filter val="P0"/>
+        <filter val="P1"/>
       </filters>
     </filterColumn>
     <filterColumn colId="5">
@@ -9123,7 +9135,7 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:G49"/>
+  <dimension ref="A1:G50"/>
   <sheetFormatPr defaultColWidth="10" defaultRowHeight="13.5" outlineLevelCol="6"/>
   <sheetData>
     <row r="1" spans="1:2">
@@ -9247,304 +9259,304 @@
         <v>702</v>
       </c>
     </row>
-    <row r="19" spans="1:2">
-      <c r="A19" t="s">
-        <v>703</v>
-      </c>
-    </row>
     <row r="20" spans="1:2">
       <c r="A20" t="s">
-        <v>704</v>
-      </c>
-      <c r="B20" t="s">
-        <v>705</v>
+        <v>703</v>
       </c>
     </row>
     <row r="21" spans="1:2">
       <c r="A21" t="s">
-        <v>706</v>
+        <v>704</v>
       </c>
       <c r="B21" t="s">
-        <v>707</v>
+        <v>705</v>
       </c>
     </row>
     <row r="22" spans="1:2">
       <c r="A22" t="s">
-        <v>708</v>
+        <v>706</v>
       </c>
       <c r="B22" t="s">
-        <v>709</v>
+        <v>707</v>
       </c>
     </row>
     <row r="23" spans="1:2">
       <c r="A23" t="s">
-        <v>710</v>
+        <v>708</v>
       </c>
       <c r="B23" t="s">
-        <v>711</v>
+        <v>709</v>
       </c>
     </row>
     <row r="24" spans="1:2">
       <c r="A24" t="s">
-        <v>712</v>
+        <v>710</v>
       </c>
       <c r="B24" t="s">
-        <v>713</v>
+        <v>711</v>
       </c>
     </row>
     <row r="25" spans="1:2">
       <c r="A25" t="s">
+        <v>712</v>
+      </c>
+      <c r="B25" t="s">
+        <v>713</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2">
+      <c r="A26" t="s">
         <v>714</v>
       </c>
-      <c r="B25" t="s">
+      <c r="B26" t="s">
         <v>715</v>
-      </c>
-    </row>
-    <row r="27" spans="1:2">
-      <c r="A27" t="s">
-        <v>716</v>
       </c>
     </row>
     <row r="28" spans="1:2">
       <c r="A28" t="s">
-        <v>717</v>
-      </c>
-      <c r="B28" t="s">
-        <v>718</v>
+        <v>716</v>
       </c>
     </row>
     <row r="29" spans="1:2">
       <c r="A29" t="s">
+        <v>717</v>
+      </c>
+      <c r="B29" t="s">
+        <v>718</v>
+      </c>
+    </row>
+    <row r="30" spans="1:2">
+      <c r="A30" t="s">
         <v>719</v>
       </c>
-      <c r="B29" t="s">
+      <c r="B30" t="s">
         <v>720</v>
       </c>
     </row>
-    <row r="30" spans="1:2">
-      <c r="B30" t="s">
+    <row r="31" spans="1:2">
+      <c r="B31" t="s">
         <v>721</v>
-      </c>
-    </row>
-    <row r="32" spans="1:2">
-      <c r="A32" t="s">
-        <v>722</v>
       </c>
     </row>
     <row r="33" spans="1:7">
       <c r="A33" t="s">
+        <v>722</v>
+      </c>
+    </row>
+    <row r="34" spans="1:7">
+      <c r="A34" t="s">
         <v>717</v>
       </c>
-      <c r="B33" t="s">
+      <c r="B34" t="s">
         <v>723</v>
-      </c>
-    </row>
-    <row r="34" spans="1:7">
-      <c r="B34" t="s">
-        <v>724</v>
       </c>
     </row>
     <row r="35" spans="1:7">
       <c r="B35" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
     </row>
     <row r="36" spans="1:7">
       <c r="B36" t="s">
-        <v>726</v>
+        <v>725</v>
       </c>
     </row>
     <row r="37" spans="1:7">
       <c r="B37" t="s">
+        <v>726</v>
+      </c>
+    </row>
+    <row r="38" spans="1:7">
+      <c r="B38" t="s">
         <v>727</v>
-      </c>
-    </row>
-    <row r="39" spans="1:7">
-      <c r="A39" t="s">
-        <v>728</v>
       </c>
     </row>
     <row r="40" spans="1:7">
       <c r="A40" t="s">
-        <v>729</v>
-      </c>
-      <c r="B40" t="s">
-        <v>730</v>
-      </c>
-      <c r="C40" t="s">
-        <v>21</v>
-      </c>
-      <c r="D40" t="s">
-        <v>731</v>
-      </c>
-      <c r="E40" t="s">
-        <v>732</v>
-      </c>
-      <c r="F40" t="s">
-        <v>733</v>
-      </c>
-      <c r="G40" t="s">
-        <v>734</v>
+        <v>728</v>
       </c>
     </row>
     <row r="41" spans="1:7">
       <c r="A41" t="s">
-        <v>735</v>
+        <v>729</v>
       </c>
       <c r="B41" t="s">
-        <v>736</v>
+        <v>730</v>
       </c>
       <c r="C41" t="s">
-        <v>737</v>
+        <v>21</v>
       </c>
       <c r="D41" t="s">
-        <v>738</v>
+        <v>731</v>
       </c>
       <c r="E41" t="s">
-        <v>739</v>
-      </c>
-      <c r="F41">
-        <v>40</v>
-      </c>
-      <c r="G41">
-        <v>-20</v>
+        <v>732</v>
+      </c>
+      <c r="F41" t="s">
+        <v>733</v>
+      </c>
+      <c r="G41" t="s">
+        <v>734</v>
       </c>
     </row>
     <row r="42" spans="1:7">
       <c r="A42" t="s">
-        <v>740</v>
+        <v>735</v>
       </c>
       <c r="B42" t="s">
-        <v>741</v>
+        <v>736</v>
       </c>
       <c r="C42" t="s">
-        <v>742</v>
+        <v>737</v>
       </c>
       <c r="D42" t="s">
-        <v>743</v>
+        <v>738</v>
       </c>
       <c r="E42" t="s">
-        <v>744</v>
+        <v>739</v>
       </c>
       <c r="F42">
-        <v>20</v>
+        <v>40</v>
       </c>
       <c r="G42">
-        <v>-10</v>
+        <v>-20</v>
       </c>
     </row>
     <row r="43" spans="1:7">
       <c r="A43" t="s">
+        <v>740</v>
+      </c>
+      <c r="B43" t="s">
+        <v>741</v>
+      </c>
+      <c r="C43" t="s">
+        <v>742</v>
+      </c>
+      <c r="D43" t="s">
+        <v>743</v>
+      </c>
+      <c r="E43" t="s">
+        <v>744</v>
+      </c>
+      <c r="F43">
+        <v>20</v>
+      </c>
+      <c r="G43">
+        <v>-10</v>
+      </c>
+    </row>
+    <row r="44" spans="1:7">
+      <c r="A44" t="s">
         <v>745</v>
       </c>
-      <c r="B43" t="s">
+      <c r="B44" t="s">
         <v>746</v>
       </c>
-      <c r="C43" t="s">
+      <c r="C44" t="s">
         <v>747</v>
       </c>
-      <c r="D43" t="s">
+      <c r="D44" t="s">
         <v>748</v>
       </c>
-      <c r="E43" t="s">
+      <c r="E44" t="s">
         <v>749</v>
       </c>
-      <c r="F43">
+      <c r="F44">
         <v>10</v>
       </c>
-      <c r="G43">
+      <c r="G44">
         <v>-5</v>
       </c>
     </row>
-    <row r="46" spans="1:7">
-      <c r="A46" s="6" t="s">
+    <row r="47" spans="1:7">
+      <c r="A47" s="6" t="s">
         <v>750</v>
       </c>
-      <c r="B46" t="s">
+      <c r="B47" t="s">
         <v>751</v>
       </c>
-      <c r="C46" t="s">
+      <c r="C47" t="s">
         <v>752</v>
       </c>
-      <c r="D46" t="s">
+      <c r="D47" t="s">
         <v>753</v>
       </c>
-      <c r="E46" t="s">
+      <c r="E47" t="s">
         <v>754</v>
       </c>
-      <c r="F46" t="s">
+      <c r="F47" t="s">
         <v>755</v>
       </c>
-      <c r="G46" t="s">
+      <c r="G47" t="s">
         <v>756</v>
-      </c>
-    </row>
-    <row r="47" spans="1:7">
-      <c r="A47" t="s">
-        <v>757</v>
-      </c>
-      <c r="B47" t="s">
-        <v>758</v>
-      </c>
-      <c r="C47" t="s">
-        <v>759</v>
-      </c>
-      <c r="D47" t="s">
-        <v>567</v>
-      </c>
-      <c r="E47" t="s">
-        <v>760</v>
-      </c>
-      <c r="F47" t="s">
-        <v>761</v>
-      </c>
-      <c r="G47" t="s">
-        <v>762</v>
       </c>
     </row>
     <row r="48" spans="1:7">
       <c r="A48" t="s">
-        <v>763</v>
+        <v>757</v>
       </c>
       <c r="B48" t="s">
-        <v>764</v>
+        <v>758</v>
       </c>
       <c r="C48" t="s">
-        <v>765</v>
+        <v>759</v>
       </c>
       <c r="D48" t="s">
-        <v>766</v>
+        <v>567</v>
       </c>
       <c r="E48" t="s">
-        <v>767</v>
+        <v>760</v>
       </c>
       <c r="F48" t="s">
-        <v>768</v>
+        <v>761</v>
       </c>
       <c r="G48" t="s">
-        <v>769</v>
+        <v>762</v>
       </c>
     </row>
     <row r="49" spans="1:7">
       <c r="A49" t="s">
+        <v>763</v>
+      </c>
+      <c r="B49" t="s">
+        <v>764</v>
+      </c>
+      <c r="C49" t="s">
+        <v>765</v>
+      </c>
+      <c r="D49" t="s">
+        <v>766</v>
+      </c>
+      <c r="E49" t="s">
+        <v>767</v>
+      </c>
+      <c r="F49" t="s">
+        <v>768</v>
+      </c>
+      <c r="G49" t="s">
+        <v>769</v>
+      </c>
+    </row>
+    <row r="50" spans="1:7">
+      <c r="A50" t="s">
         <v>770</v>
       </c>
-      <c r="B49" t="s">
+      <c r="B50" t="s">
         <v>771</v>
       </c>
-      <c r="C49" t="s">
+      <c r="C50" t="s">
         <v>772</v>
       </c>
-      <c r="D49" t="s">
+      <c r="D50" t="s">
         <v>773</v>
       </c>
-      <c r="E49" t="s">
+      <c r="E50" t="s">
         <v>774</v>
       </c>
-      <c r="F49" t="s">
+      <c r="F50" t="s">
         <v>775</v>
       </c>
-      <c r="G49" t="s">
+      <c r="G50" t="s">
         <v>776</v>
       </c>
     </row>
@@ -9557,7 +9569,7 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:H37"/>
+  <dimension ref="A1:H38"/>
   <sheetFormatPr defaultColWidth="10" defaultRowHeight="13.5" outlineLevelCol="7"/>
   <cols>
     <col min="2" max="2" width="15.7" customWidth="1"/>
@@ -9759,129 +9771,114 @@
     </row>
     <row r="28" spans="1:3">
       <c r="A28" s="2" t="s">
+        <v>794</v>
+      </c>
+      <c r="B28" s="2" t="s">
         <v>812</v>
       </c>
-      <c r="B28" s="2" t="s">
+      <c r="C28" s="2" t="s">
         <v>813</v>
-      </c>
-      <c r="C28" s="2" t="s">
-        <v>814</v>
       </c>
     </row>
     <row r="29" spans="1:3">
       <c r="A29" s="2" t="s">
+        <v>814</v>
+      </c>
+      <c r="B29" s="2" t="s">
         <v>815</v>
       </c>
-      <c r="B29" s="2" t="s">
+      <c r="C29" s="2" t="s">
         <v>816</v>
       </c>
-      <c r="C29" s="2" t="s">
+    </row>
+    <row r="30" spans="1:3">
+      <c r="A30" s="2" t="s">
         <v>817</v>
       </c>
-    </row>
-    <row r="30" spans="1:3">
-      <c r="A30" s="4" t="s">
+      <c r="B30" s="2" t="s">
         <v>818</v>
       </c>
-      <c r="B30" s="4" t="s">
+      <c r="C30" s="2" t="s">
         <v>819</v>
       </c>
-      <c r="C30" s="4" t="s">
+    </row>
+    <row r="31" spans="1:3">
+      <c r="A31" s="4" t="s">
         <v>820</v>
       </c>
-    </row>
-    <row r="31" spans="1:3">
-      <c r="A31" s="2" t="s">
+      <c r="B31" s="4" t="s">
         <v>821</v>
       </c>
-      <c r="B31" s="2" t="s">
+      <c r="C31" s="4" t="s">
         <v>822</v>
-      </c>
-      <c r="C31" s="2" t="s">
-        <v>823</v>
       </c>
     </row>
     <row r="32" spans="1:3">
       <c r="A32" s="2" t="s">
+        <v>823</v>
+      </c>
+      <c r="B32" s="2" t="s">
         <v>824</v>
       </c>
-      <c r="B32" s="2" t="s">
+      <c r="C32" s="2" t="s">
         <v>825</v>
       </c>
-      <c r="C32" s="2" t="s">
+    </row>
+    <row r="33" spans="1:8">
+      <c r="A33" s="2" t="s">
         <v>826</v>
       </c>
-    </row>
-    <row r="34" spans="1:8">
-      <c r="A34" s="2" t="s">
-        <v>729</v>
-      </c>
-      <c r="B34" s="2" t="s">
+      <c r="B33" s="2" t="s">
         <v>827</v>
       </c>
-      <c r="C34" s="2" t="s">
+      <c r="C33" s="2" t="s">
         <v>828</v>
-      </c>
-      <c r="D34" s="2" t="s">
-        <v>829</v>
-      </c>
-      <c r="E34" s="2" t="s">
-        <v>830</v>
-      </c>
-      <c r="F34" s="2" t="s">
-        <v>831</v>
-      </c>
-      <c r="G34" s="2" t="s">
-        <v>787</v>
-      </c>
-      <c r="H34" s="2" t="s">
-        <v>788</v>
       </c>
     </row>
     <row r="35" spans="1:8">
       <c r="A35" s="2" t="s">
-        <v>735</v>
+        <v>729</v>
       </c>
       <c r="B35" s="2" t="s">
-        <v>789</v>
+        <v>829</v>
       </c>
       <c r="C35" s="2" t="s">
+        <v>830</v>
+      </c>
+      <c r="D35" s="2" t="s">
+        <v>831</v>
+      </c>
+      <c r="E35" s="2" t="s">
         <v>832</v>
       </c>
-      <c r="D35" s="2" t="s">
-        <v>809</v>
-      </c>
-      <c r="E35" s="2" t="s">
-        <v>818</v>
-      </c>
-      <c r="F35" s="2">
-        <v>40</v>
-      </c>
-      <c r="G35" s="5">
-        <v>0.5</v>
-      </c>
-      <c r="H35" s="5">
-        <v>-0.5</v>
+      <c r="F35" s="2" t="s">
+        <v>833</v>
+      </c>
+      <c r="G35" s="2" t="s">
+        <v>787</v>
+      </c>
+      <c r="H35" s="2" t="s">
+        <v>788</v>
       </c>
     </row>
     <row r="36" spans="1:8">
       <c r="A36" s="2" t="s">
-        <v>740</v>
+        <v>735</v>
       </c>
       <c r="B36" s="2" t="s">
-        <v>833</v>
+        <v>789</v>
       </c>
       <c r="C36" s="2" t="s">
         <v>834</v>
       </c>
       <c r="D36" s="2" t="s">
-        <v>812</v>
+        <v>794</v>
       </c>
       <c r="E36" s="2" t="s">
-        <v>821</v>
+        <v>820</v>
       </c>
       <c r="F36" s="2">
-        <v>20</v>
+        <v>40</v>
       </c>
       <c r="G36" s="5">
         <v>0.5</v>
@@ -9892,27 +9889,53 @@
     </row>
     <row r="37" spans="1:8">
       <c r="A37" s="2" t="s">
+        <v>740</v>
+      </c>
+      <c r="B37" s="2" t="s">
         <v>835</v>
       </c>
-      <c r="B37" s="2" t="s">
+      <c r="C37" s="2" t="s">
         <v>836</v>
       </c>
-      <c r="C37" s="2" t="s">
-        <v>806</v>
-      </c>
       <c r="D37" s="2" t="s">
-        <v>815</v>
+        <v>814</v>
       </c>
       <c r="E37" s="2" t="s">
-        <v>824</v>
+        <v>823</v>
       </c>
       <c r="F37" s="2">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="G37" s="5">
         <v>0.5</v>
       </c>
       <c r="H37" s="5">
+        <v>-0.5</v>
+      </c>
+    </row>
+    <row r="38" spans="1:8">
+      <c r="A38" s="2" t="s">
+        <v>837</v>
+      </c>
+      <c r="B38" s="2" t="s">
+        <v>838</v>
+      </c>
+      <c r="C38" s="2" t="s">
+        <v>809</v>
+      </c>
+      <c r="D38" s="2" t="s">
+        <v>817</v>
+      </c>
+      <c r="E38" s="2" t="s">
+        <v>826</v>
+      </c>
+      <c r="F38" s="2">
+        <v>10</v>
+      </c>
+      <c r="G38" s="5">
+        <v>0.5</v>
+      </c>
+      <c r="H38" s="5">
         <v>-0.5</v>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: update GUI product planning docs
</commit_message>
<xml_diff>
--- a/docs/MVP 0.9 项目管理/01_需求与版本规划/EOR MVP 1.0 目标版本规划 V1.1.xlsx
+++ b/docs/MVP 0.9 项目管理/01_需求与版本规划/EOR MVP 1.0 目标版本规划 V1.1.xlsx
@@ -1390,6 +1390,12 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Segoe UI"/>
+        <charset val="134"/>
+      </rPr>
       <t xml:space="preserve">P0 </t>
     </r>
     <r>
@@ -4376,6 +4382,9 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -4404,9 +4413,6 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1">
@@ -4710,7 +4716,7 @@
     </dxf>
   </dxfs>
   <tableStyles count="2" defaultTableStyle="TableStylePreset3_Accent1 1" defaultPivotStyle="PivotStylePreset2_Accent1 1">
-    <tableStyle name="TableStylePreset3_Accent1 1" pivot="0" count="7" xr9:uid="{DCD53CD2-7D63-465F-8282-B831EBB5EED1}">
+    <tableStyle name="TableStylePreset3_Accent1 1" pivot="0" count="7" xr9:uid="{02CC191A-CB85-447D-A12E-4AD26D929F4B}">
       <tableStyleElement type="wholeTable" dxfId="7"/>
       <tableStyleElement type="headerRow" dxfId="6"/>
       <tableStyleElement type="totalRow" dxfId="5"/>
@@ -4719,7 +4725,7 @@
       <tableStyleElement type="firstRowStripe" dxfId="2"/>
       <tableStyleElement type="firstColumnStripe" dxfId="1"/>
     </tableStyle>
-    <tableStyle name="PivotStylePreset2_Accent1 1" table="0" count="10" xr9:uid="{D209FF72-8775-4799-A746-0B9339E74356}">
+    <tableStyle name="PivotStylePreset2_Accent1 1" table="0" count="10" xr9:uid="{4C31328B-8DBA-47F9-B89D-1D92FC4E42C7}">
       <tableStyleElement type="headerRow" dxfId="17"/>
       <tableStyleElement type="totalRow" dxfId="16"/>
       <tableStyleElement type="firstRowStripe" dxfId="15"/>
@@ -5334,7 +5340,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr filterMode="1"/>
+  <sheetPr/>
   <dimension ref="A1:G114"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5" outlineLevelCol="6"/>
   <cols>
@@ -5385,7 +5391,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="4" ht="19.5" hidden="1" spans="1:7">
+    <row r="4" ht="19.5" spans="1:7">
       <c r="A4" s="2"/>
       <c r="B4" s="25" t="s">
         <v>73</v>
@@ -5398,7 +5404,7 @@
       <c r="F4" s="2"/>
       <c r="G4" s="2"/>
     </row>
-    <row r="5" ht="30" hidden="1" spans="1:7">
+    <row r="5" ht="30" spans="1:7">
       <c r="A5" s="2" t="s">
         <v>75</v>
       </c>
@@ -5414,7 +5420,7 @@
       <c r="E5" s="27" t="s">
         <v>79</v>
       </c>
-      <c r="F5" s="2" t="s">
+      <c r="F5" s="30" t="s">
         <v>80</v>
       </c>
       <c r="G5" s="2"/>
@@ -5440,7 +5446,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" ht="27" hidden="1" spans="1:7">
+    <row r="7" ht="27" spans="1:7">
       <c r="A7" s="2"/>
       <c r="B7" s="2" t="s">
         <v>85</v>
@@ -5499,7 +5505,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="10" ht="27" hidden="1" spans="1:7">
+    <row r="10" ht="27" spans="1:7">
       <c r="A10" s="2" t="s">
         <v>96</v>
       </c>
@@ -5512,7 +5518,7 @@
       <c r="D10" s="26" t="s">
         <v>98</v>
       </c>
-      <c r="E10" s="30" t="s">
+      <c r="E10" s="31" t="s">
         <v>99</v>
       </c>
       <c r="F10" s="2"/>
@@ -5520,7 +5526,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="11" ht="40.5" hidden="1" spans="1:7">
+    <row r="11" ht="40.5" spans="1:7">
       <c r="A11" s="2"/>
       <c r="B11" s="2" t="s">
         <v>100</v>
@@ -5537,7 +5543,7 @@
       <c r="F11" s="2"/>
       <c r="G11" s="2"/>
     </row>
-    <row r="12" ht="27" hidden="1" spans="1:7">
+    <row r="12" ht="27" spans="1:7">
       <c r="A12" s="2"/>
       <c r="B12" s="2" t="s">
         <v>103</v>
@@ -5554,7 +5560,7 @@
       <c r="F12" s="2"/>
       <c r="G12" s="2"/>
     </row>
-    <row r="13" ht="40.5" hidden="1" spans="1:7">
+    <row r="13" ht="40.5" spans="1:7">
       <c r="A13" s="2"/>
       <c r="B13" s="2" t="s">
         <v>106</v>
@@ -5571,7 +5577,7 @@
       <c r="F13" s="2"/>
       <c r="G13" s="2"/>
     </row>
-    <row r="14" ht="27" hidden="1" spans="1:7">
+    <row r="14" ht="27" spans="1:7">
       <c r="A14" s="2" t="s">
         <v>109</v>
       </c>
@@ -5584,7 +5590,7 @@
       <c r="D14" s="27" t="s">
         <v>111</v>
       </c>
-      <c r="E14" s="30" t="s">
+      <c r="E14" s="31" t="s">
         <v>99</v>
       </c>
       <c r="F14" s="2"/>
@@ -5592,7 +5598,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="15" ht="27" hidden="1" spans="1:7">
+    <row r="15" ht="27" spans="1:7">
       <c r="A15" s="2"/>
       <c r="B15" s="27" t="s">
         <v>112</v>
@@ -5609,7 +5615,7 @@
       <c r="F15" s="2"/>
       <c r="G15" s="2"/>
     </row>
-    <row r="16" ht="108" hidden="1" spans="1:7">
+    <row r="16" ht="108" spans="1:7">
       <c r="A16" s="2"/>
       <c r="B16" s="2" t="s">
         <v>115</v>
@@ -5626,7 +5632,7 @@
       <c r="F16" s="2"/>
       <c r="G16" s="2"/>
     </row>
-    <row r="17" ht="19.5" hidden="1" spans="1:7">
+    <row r="17" ht="19.5" spans="1:7">
       <c r="A17" s="2"/>
       <c r="B17" s="25" t="s">
         <v>119</v>
@@ -5639,11 +5645,11 @@
       <c r="F17" s="2"/>
       <c r="G17" s="2"/>
     </row>
-    <row r="18" ht="40.5" hidden="1" spans="1:7">
+    <row r="18" ht="40.5" spans="1:7">
       <c r="A18" s="2" t="s">
         <v>120</v>
       </c>
-      <c r="B18" s="31" t="s">
+      <c r="B18" s="32" t="s">
         <v>121</v>
       </c>
       <c r="C18" s="29" t="s">
@@ -5655,16 +5661,16 @@
       <c r="E18" s="27" t="s">
         <v>79</v>
       </c>
-      <c r="F18" s="2" t="s">
+      <c r="F18" s="30" t="s">
         <v>80</v>
       </c>
       <c r="G18" s="2"/>
     </row>
-    <row r="19" ht="30" hidden="1" spans="1:7">
+    <row r="19" ht="30" spans="1:7">
       <c r="A19" s="2" t="s">
         <v>124</v>
       </c>
-      <c r="B19" s="31" t="s">
+      <c r="B19" s="32" t="s">
         <v>125</v>
       </c>
       <c r="C19" s="29" t="s">
@@ -5676,12 +5682,12 @@
       <c r="E19" s="27" t="s">
         <v>79</v>
       </c>
-      <c r="F19" s="2" t="s">
+      <c r="F19" s="30" t="s">
         <v>80</v>
       </c>
       <c r="G19" s="2"/>
     </row>
-    <row r="20" ht="46.5" hidden="1" spans="1:7">
+    <row r="20" ht="46.5" spans="1:7">
       <c r="A20" s="2" t="s">
         <v>128</v>
       </c>
@@ -5697,16 +5703,16 @@
       <c r="E20" s="27" t="s">
         <v>79</v>
       </c>
-      <c r="F20" s="2" t="s">
+      <c r="F20" s="30" t="s">
         <v>80</v>
       </c>
       <c r="G20" s="2"/>
     </row>
-    <row r="21" ht="40.5" hidden="1" spans="1:7">
+    <row r="21" ht="40.5" spans="1:7">
       <c r="A21" s="2" t="s">
         <v>132</v>
       </c>
-      <c r="B21" s="31" t="s">
+      <c r="B21" s="32" t="s">
         <v>133</v>
       </c>
       <c r="C21" s="29" t="s">
@@ -5718,12 +5724,12 @@
       <c r="E21" s="27" t="s">
         <v>79</v>
       </c>
-      <c r="F21" s="2" t="s">
+      <c r="F21" s="30" t="s">
         <v>80</v>
       </c>
       <c r="G21" s="2"/>
     </row>
-    <row r="22" ht="40.5" hidden="1" spans="1:7">
+    <row r="22" ht="40.5" spans="1:7">
       <c r="A22" s="2" t="s">
         <v>136</v>
       </c>
@@ -5736,7 +5742,7 @@
       <c r="D22" s="26" t="s">
         <v>138</v>
       </c>
-      <c r="E22" s="30" t="s">
+      <c r="E22" s="31" t="s">
         <v>99</v>
       </c>
       <c r="F22" s="2"/>
@@ -5744,7 +5750,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="23" ht="27" hidden="1" spans="1:7">
+    <row r="23" ht="27" spans="1:7">
       <c r="A23" s="2"/>
       <c r="B23" s="2" t="s">
         <v>139</v>
@@ -5761,7 +5767,7 @@
       <c r="F23" s="2"/>
       <c r="G23" s="2"/>
     </row>
-    <row r="24" ht="27" hidden="1" spans="1:7">
+    <row r="24" ht="27" spans="1:7">
       <c r="A24" s="2"/>
       <c r="B24" s="27" t="s">
         <v>142</v>
@@ -5778,7 +5784,7 @@
       <c r="F24" s="2"/>
       <c r="G24" s="2"/>
     </row>
-    <row r="25" ht="27" hidden="1" spans="1:7">
+    <row r="25" ht="27" spans="1:7">
       <c r="A25" s="2"/>
       <c r="B25" s="27" t="s">
         <v>145</v>
@@ -5795,7 +5801,7 @@
       <c r="F25" s="2"/>
       <c r="G25" s="2"/>
     </row>
-    <row r="26" ht="27" hidden="1" spans="1:7">
+    <row r="26" ht="27" spans="1:7">
       <c r="A26" s="2"/>
       <c r="B26" s="2" t="s">
         <v>147</v>
@@ -5812,7 +5818,7 @@
       <c r="F26" s="2"/>
       <c r="G26" s="2"/>
     </row>
-    <row r="27" ht="43.5" hidden="1" spans="1:7">
+    <row r="27" ht="43.5" spans="1:7">
       <c r="A27" s="2" t="s">
         <v>150</v>
       </c>
@@ -5825,7 +5831,7 @@
       <c r="D27" s="29" t="s">
         <v>153</v>
       </c>
-      <c r="E27" s="30" t="s">
+      <c r="E27" s="31" t="s">
         <v>99</v>
       </c>
       <c r="F27" s="2"/>
@@ -5833,7 +5839,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="28" ht="16.5" hidden="1" spans="1:7">
+    <row r="28" ht="16.5" spans="1:7">
       <c r="A28" s="2"/>
       <c r="B28" s="2" t="s">
         <v>154</v>
@@ -5850,11 +5856,11 @@
       <c r="F28" s="2"/>
       <c r="G28" s="2"/>
     </row>
-    <row r="29" ht="30" hidden="1" spans="1:7">
+    <row r="29" ht="30" spans="1:7">
       <c r="A29" s="2" t="s">
         <v>157</v>
       </c>
-      <c r="B29" s="32" t="s">
+      <c r="B29" s="33" t="s">
         <v>158</v>
       </c>
       <c r="C29" s="29" t="s">
@@ -5863,7 +5869,7 @@
       <c r="D29" s="27" t="s">
         <v>160</v>
       </c>
-      <c r="E29" s="30" t="s">
+      <c r="E29" s="31" t="s">
         <v>99</v>
       </c>
       <c r="F29" s="2"/>
@@ -5871,11 +5877,11 @@
         <v>8</v>
       </c>
     </row>
-    <row r="30" ht="43.5" hidden="1" spans="1:7">
+    <row r="30" ht="43.5" spans="1:7">
       <c r="A30" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="B30" s="32" t="s">
+      <c r="B30" s="33" t="s">
         <v>162</v>
       </c>
       <c r="C30" s="29" t="s">
@@ -5892,7 +5898,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="31" customFormat="1" ht="54" hidden="1" spans="1:7">
+    <row r="31" customFormat="1" ht="54" spans="1:7">
       <c r="A31" s="2"/>
       <c r="B31" s="2" t="s">
         <v>164</v>
@@ -5909,7 +5915,7 @@
       <c r="F31" s="2"/>
       <c r="G31" s="2"/>
     </row>
-    <row r="32" ht="19.5" hidden="1" spans="1:7">
+    <row r="32" ht="19.5" spans="1:7">
       <c r="A32" s="2"/>
       <c r="B32" s="25" t="s">
         <v>167</v>
@@ -5922,7 +5928,7 @@
       <c r="F32" s="2"/>
       <c r="G32" s="2"/>
     </row>
-    <row r="33" ht="40.5" hidden="1" spans="1:7">
+    <row r="33" ht="40.5" spans="1:7">
       <c r="A33" s="2"/>
       <c r="B33" s="2" t="s">
         <v>168</v>
@@ -5939,11 +5945,11 @@
       <c r="F33" s="2"/>
       <c r="G33" s="2"/>
     </row>
-    <row r="34" ht="33" hidden="1" spans="1:7">
+    <row r="34" ht="33" spans="1:7">
       <c r="A34" s="2" t="s">
         <v>171</v>
       </c>
-      <c r="B34" s="31" t="s">
+      <c r="B34" s="32" t="s">
         <v>172</v>
       </c>
       <c r="C34" s="29" t="s">
@@ -5955,12 +5961,12 @@
       <c r="E34" s="27" t="s">
         <v>79</v>
       </c>
-      <c r="F34" s="2" t="s">
+      <c r="F34" s="30" t="s">
         <v>80</v>
       </c>
       <c r="G34" s="2"/>
     </row>
-    <row r="35" ht="43.5" hidden="1" spans="1:7">
+    <row r="35" ht="43.5" spans="1:7">
       <c r="A35" s="2" t="s">
         <v>175</v>
       </c>
@@ -5976,16 +5982,16 @@
       <c r="E35" s="27" t="s">
         <v>79</v>
       </c>
-      <c r="F35" s="2" t="s">
+      <c r="F35" s="30" t="s">
         <v>80</v>
       </c>
       <c r="G35" s="2"/>
     </row>
-    <row r="36" ht="27" hidden="1" spans="1:7">
+    <row r="36" ht="27" spans="1:7">
       <c r="A36" s="2" t="s">
         <v>179</v>
       </c>
-      <c r="B36" s="32" t="s">
+      <c r="B36" s="33" t="s">
         <v>180</v>
       </c>
       <c r="C36" s="29" t="s">
@@ -6002,7 +6008,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="37" customFormat="1" ht="57" hidden="1" spans="1:7">
+    <row r="37" customFormat="1" ht="57" spans="1:7">
       <c r="A37" s="2"/>
       <c r="B37" s="27" t="s">
         <v>183</v>
@@ -6019,7 +6025,7 @@
       <c r="F37" s="2"/>
       <c r="G37" s="2"/>
     </row>
-    <row r="38" ht="54" hidden="1" spans="1:7">
+    <row r="38" ht="54" spans="1:7">
       <c r="A38" s="2" t="s">
         <v>185</v>
       </c>
@@ -6035,12 +6041,12 @@
       <c r="E38" s="27" t="s">
         <v>79</v>
       </c>
-      <c r="F38" s="2" t="s">
+      <c r="F38" s="30" t="s">
         <v>80</v>
       </c>
       <c r="G38" s="2"/>
     </row>
-    <row r="39" ht="81" hidden="1" spans="1:7">
+    <row r="39" ht="81" spans="1:7">
       <c r="A39" s="2"/>
       <c r="B39" s="29" t="s">
         <v>188</v>
@@ -6057,7 +6063,7 @@
       <c r="F39" s="2"/>
       <c r="G39" s="2"/>
     </row>
-    <row r="40" customFormat="1" ht="67.5" hidden="1" spans="1:7">
+    <row r="40" customFormat="1" ht="67.5" spans="1:7">
       <c r="A40" s="2"/>
       <c r="B40" s="2" t="s">
         <v>191</v>
@@ -6074,7 +6080,7 @@
       <c r="F40" s="2"/>
       <c r="G40" s="2"/>
     </row>
-    <row r="41" customFormat="1" ht="27" hidden="1" spans="1:7">
+    <row r="41" customFormat="1" ht="27" spans="1:7">
       <c r="A41" s="2"/>
       <c r="B41" s="2" t="s">
         <v>194</v>
@@ -6091,7 +6097,7 @@
       <c r="F41" s="2"/>
       <c r="G41" s="2"/>
     </row>
-    <row r="42" customFormat="1" ht="16.5" hidden="1" spans="1:7">
+    <row r="42" customFormat="1" ht="16.5" spans="1:7">
       <c r="A42" s="2"/>
       <c r="B42" s="2" t="s">
         <v>197</v>
@@ -6108,7 +6114,7 @@
       <c r="F42" s="2"/>
       <c r="G42" s="2"/>
     </row>
-    <row r="43" customFormat="1" ht="67.5" hidden="1" spans="1:7">
+    <row r="43" customFormat="1" ht="67.5" spans="1:7">
       <c r="A43" s="2"/>
       <c r="B43" s="2" t="s">
         <v>200</v>
@@ -6125,7 +6131,7 @@
       <c r="F43" s="2"/>
       <c r="G43" s="2"/>
     </row>
-    <row r="44" customFormat="1" ht="54" hidden="1" spans="1:7">
+    <row r="44" customFormat="1" ht="54" spans="1:7">
       <c r="A44" s="2"/>
       <c r="B44" s="2" t="s">
         <v>203</v>
@@ -6142,7 +6148,7 @@
       <c r="F44" s="2"/>
       <c r="G44" s="2"/>
     </row>
-    <row r="45" customFormat="1" ht="67.5" hidden="1" spans="1:7">
+    <row r="45" customFormat="1" ht="67.5" spans="1:7">
       <c r="A45" s="2"/>
       <c r="B45" s="2" t="s">
         <v>206</v>
@@ -6159,7 +6165,7 @@
       <c r="F45" s="2"/>
       <c r="G45" s="2"/>
     </row>
-    <row r="46" ht="24" hidden="1" spans="1:7">
+    <row r="46" ht="24" spans="1:7">
       <c r="A46" s="2"/>
       <c r="B46" s="25" t="s">
         <v>209</v>
@@ -6172,7 +6178,7 @@
       <c r="F46" s="2"/>
       <c r="G46" s="2"/>
     </row>
-    <row r="47" ht="16.5" hidden="1" spans="1:7">
+    <row r="47" ht="16.5" spans="1:7">
       <c r="A47" s="2" t="s">
         <v>210</v>
       </c>
@@ -6188,16 +6194,16 @@
       <c r="E47" s="27" t="s">
         <v>79</v>
       </c>
-      <c r="F47" s="2" t="s">
+      <c r="F47" s="30" t="s">
         <v>80</v>
       </c>
       <c r="G47" s="2"/>
     </row>
-    <row r="48" ht="30" hidden="1" spans="1:7">
+    <row r="48" ht="30" spans="1:7">
       <c r="A48" s="2" t="s">
         <v>214</v>
       </c>
-      <c r="B48" s="31" t="s">
+      <c r="B48" s="32" t="s">
         <v>215</v>
       </c>
       <c r="C48" s="29" t="s">
@@ -6209,12 +6215,12 @@
       <c r="E48" s="27" t="s">
         <v>79</v>
       </c>
-      <c r="F48" s="2" t="s">
+      <c r="F48" s="30" t="s">
         <v>80</v>
       </c>
       <c r="G48" s="2"/>
     </row>
-    <row r="49" ht="27" hidden="1" spans="1:7">
+    <row r="49" ht="27" spans="1:7">
       <c r="A49" s="2" t="s">
         <v>218</v>
       </c>
@@ -6230,12 +6236,12 @@
       <c r="E49" s="27" t="s">
         <v>79</v>
       </c>
-      <c r="F49" s="2" t="s">
+      <c r="F49" s="30" t="s">
         <v>80</v>
       </c>
       <c r="G49" s="2"/>
     </row>
-    <row r="50" ht="16.5" hidden="1" spans="1:7">
+    <row r="50" ht="16.5" spans="1:7">
       <c r="A50" s="2" t="s">
         <v>222</v>
       </c>
@@ -6251,12 +6257,12 @@
       <c r="E50" s="27" t="s">
         <v>79</v>
       </c>
-      <c r="F50" s="2" t="s">
+      <c r="F50" s="30" t="s">
         <v>80</v>
       </c>
       <c r="G50" s="2"/>
     </row>
-    <row r="51" ht="16.5" hidden="1" spans="1:7">
+    <row r="51" ht="16.5" spans="1:7">
       <c r="A51" s="2"/>
       <c r="B51" s="2" t="s">
         <v>226</v>
@@ -6273,7 +6279,7 @@
       <c r="F51" s="2"/>
       <c r="G51" s="2"/>
     </row>
-    <row r="52" ht="27" hidden="1" spans="1:7">
+    <row r="52" ht="27" spans="1:7">
       <c r="A52" s="2"/>
       <c r="B52" s="2" t="s">
         <v>229</v>
@@ -6290,7 +6296,7 @@
       <c r="F52" s="2"/>
       <c r="G52" s="2"/>
     </row>
-    <row r="53" ht="27" hidden="1" spans="1:7">
+    <row r="53" ht="27" spans="1:7">
       <c r="A53" s="2"/>
       <c r="B53" s="2" t="s">
         <v>232</v>
@@ -6307,7 +6313,7 @@
       <c r="F53" s="2"/>
       <c r="G53" s="2"/>
     </row>
-    <row r="54" ht="27" hidden="1" spans="1:7">
+    <row r="54" ht="27" spans="1:7">
       <c r="A54" s="2"/>
       <c r="B54" s="2" t="s">
         <v>235</v>
@@ -6324,7 +6330,7 @@
       <c r="F54" s="2"/>
       <c r="G54" s="2"/>
     </row>
-    <row r="55" ht="19.5" hidden="1" spans="1:7">
+    <row r="55" ht="19.5" spans="1:7">
       <c r="A55" s="2"/>
       <c r="B55" s="25" t="s">
         <v>237</v>
@@ -6337,11 +6343,11 @@
       <c r="F55" s="2"/>
       <c r="G55" s="2"/>
     </row>
-    <row r="56" ht="16.5" hidden="1" spans="1:7">
+    <row r="56" ht="16.5" spans="1:7">
       <c r="A56" s="2" t="s">
         <v>238</v>
       </c>
-      <c r="B56" s="32" t="s">
+      <c r="B56" s="33" t="s">
         <v>239</v>
       </c>
       <c r="C56" s="29" t="s">
@@ -6358,11 +6364,11 @@
         <v>11</v>
       </c>
     </row>
-    <row r="57" ht="27" hidden="1" spans="1:7">
+    <row r="57" ht="27" spans="1:7">
       <c r="A57" s="2" t="s">
         <v>241</v>
       </c>
-      <c r="B57" s="33" t="s">
+      <c r="B57" s="34" t="s">
         <v>242</v>
       </c>
       <c r="C57" s="2" t="s">
@@ -6379,7 +6385,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="58" ht="40.5" hidden="1" spans="1:7">
+    <row r="58" ht="40.5" spans="1:7">
       <c r="A58" s="2"/>
       <c r="B58" s="2" t="s">
         <v>245</v>
@@ -6396,11 +6402,11 @@
       <c r="F58" s="2"/>
       <c r="G58" s="2"/>
     </row>
-    <row r="59" ht="40.5" hidden="1" spans="1:7">
+    <row r="59" ht="40.5" spans="1:7">
       <c r="A59" s="2" t="s">
         <v>248</v>
       </c>
-      <c r="B59" s="33" t="s">
+      <c r="B59" s="34" t="s">
         <v>249</v>
       </c>
       <c r="C59" s="2" t="s">
@@ -6417,11 +6423,11 @@
         <v>13</v>
       </c>
     </row>
-    <row r="60" ht="27" hidden="1" spans="1:7">
+    <row r="60" ht="27" spans="1:7">
       <c r="A60" s="2" t="s">
         <v>252</v>
       </c>
-      <c r="B60" s="33" t="s">
+      <c r="B60" s="34" t="s">
         <v>253</v>
       </c>
       <c r="C60" s="2" t="s">
@@ -6438,11 +6444,11 @@
         <v>14</v>
       </c>
     </row>
-    <row r="61" ht="16.5" hidden="1" spans="1:7">
+    <row r="61" ht="16.5" spans="1:7">
       <c r="A61" s="2" t="s">
         <v>255</v>
       </c>
-      <c r="B61" s="33" t="s">
+      <c r="B61" s="34" t="s">
         <v>256</v>
       </c>
       <c r="C61" s="2" t="s">
@@ -6459,7 +6465,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="62" ht="19.5" hidden="1" spans="1:7">
+    <row r="62" ht="19.5" spans="1:7">
       <c r="A62" s="2"/>
       <c r="B62" s="25" t="s">
         <v>259</v>
@@ -6472,11 +6478,11 @@
       <c r="F62" s="2"/>
       <c r="G62" s="2"/>
     </row>
-    <row r="63" ht="16.5" hidden="1" spans="1:7">
+    <row r="63" ht="16.5" spans="1:7">
       <c r="A63" s="2" t="s">
         <v>260</v>
       </c>
-      <c r="B63" s="34" t="s">
+      <c r="B63" s="35" t="s">
         <v>261</v>
       </c>
       <c r="C63" s="2" t="s">
@@ -6488,16 +6494,16 @@
       <c r="E63" s="27" t="s">
         <v>79</v>
       </c>
-      <c r="F63" s="2" t="s">
+      <c r="F63" s="30" t="s">
         <v>80</v>
       </c>
       <c r="G63" s="2"/>
     </row>
-    <row r="64" ht="27" hidden="1" spans="1:7">
+    <row r="64" ht="27" spans="1:7">
       <c r="A64" s="2" t="s">
         <v>264</v>
       </c>
-      <c r="B64" s="32" t="s">
+      <c r="B64" s="33" t="s">
         <v>265</v>
       </c>
       <c r="C64" s="29" t="s">
@@ -6514,7 +6520,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="65" ht="33" hidden="1" spans="1:7">
+    <row r="65" ht="33" spans="1:7">
       <c r="A65" s="2" t="s">
         <v>268</v>
       </c>
@@ -6530,16 +6536,16 @@
       <c r="E65" s="27" t="s">
         <v>79</v>
       </c>
-      <c r="F65" s="2" t="s">
+      <c r="F65" s="30" t="s">
         <v>80</v>
       </c>
       <c r="G65" s="2"/>
     </row>
-    <row r="66" ht="43.5" hidden="1" spans="1:7">
+    <row r="66" ht="43.5" spans="1:7">
       <c r="A66" s="2" t="s">
         <v>272</v>
       </c>
-      <c r="B66" s="32" t="s">
+      <c r="B66" s="33" t="s">
         <v>273</v>
       </c>
       <c r="C66" s="29" t="s">
@@ -6556,7 +6562,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="67" ht="30" hidden="1" spans="1:7">
+    <row r="67" ht="30" spans="1:7">
       <c r="A67" s="2" t="s">
         <v>276</v>
       </c>
@@ -6572,12 +6578,12 @@
       <c r="E67" s="27" t="s">
         <v>79</v>
       </c>
-      <c r="F67" s="2" t="s">
+      <c r="F67" s="30" t="s">
         <v>80</v>
       </c>
       <c r="G67" s="2"/>
     </row>
-    <row r="68" ht="76.5" hidden="1" spans="1:7">
+    <row r="68" ht="76.5" spans="1:7">
       <c r="A68" s="2" t="s">
         <v>279</v>
       </c>
@@ -6593,12 +6599,12 @@
       <c r="E68" s="27" t="s">
         <v>79</v>
       </c>
-      <c r="F68" s="2" t="s">
+      <c r="F68" s="30" t="s">
         <v>80</v>
       </c>
       <c r="G68" s="2"/>
     </row>
-    <row r="69" ht="40.5" hidden="1" spans="1:7">
+    <row r="69" ht="40.5" spans="1:7">
       <c r="A69" s="2"/>
       <c r="B69" s="2" t="s">
         <v>282</v>
@@ -6615,11 +6621,11 @@
       <c r="F69" s="2"/>
       <c r="G69" s="2"/>
     </row>
-    <row r="70" ht="54" hidden="1" spans="1:7">
+    <row r="70" ht="54" spans="1:7">
       <c r="A70" s="2" t="s">
         <v>285</v>
       </c>
-      <c r="B70" s="33" t="s">
+      <c r="B70" s="34" t="s">
         <v>286</v>
       </c>
       <c r="C70" s="2" t="s">
@@ -6636,7 +6642,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="71" ht="40.5" hidden="1" spans="1:7">
+    <row r="71" ht="40.5" spans="1:7">
       <c r="A71" s="2" t="s">
         <v>289</v>
       </c>
@@ -6657,7 +6663,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="72" ht="27" hidden="1" spans="1:7">
+    <row r="72" ht="27" spans="1:7">
       <c r="A72" s="2" t="s">
         <v>293</v>
       </c>
@@ -6673,7 +6679,7 @@
       <c r="E72" s="27" t="s">
         <v>79</v>
       </c>
-      <c r="F72" s="2" t="s">
+      <c r="F72" s="30" t="s">
         <v>80</v>
       </c>
       <c r="G72" s="2"/>
@@ -6682,7 +6688,7 @@
       <c r="A73" s="2" t="s">
         <v>297</v>
       </c>
-      <c r="B73" s="35" t="s">
+      <c r="B73" s="36" t="s">
         <v>298</v>
       </c>
       <c r="C73" s="27" t="s">
@@ -6697,9 +6703,9 @@
       <c r="F73" s="2"/>
       <c r="G73" s="2"/>
     </row>
-    <row r="74" ht="19.5" hidden="1" spans="1:7">
+    <row r="74" ht="19.5" spans="1:7">
       <c r="A74" s="2"/>
-      <c r="B74" s="36" t="s">
+      <c r="B74" s="37" t="s">
         <v>300</v>
       </c>
       <c r="C74" s="2"/>
@@ -6710,7 +6716,7 @@
       <c r="F74" s="2"/>
       <c r="G74" s="2"/>
     </row>
-    <row r="75" ht="30" hidden="1" spans="1:7">
+    <row r="75" ht="30" spans="1:7">
       <c r="A75" s="2"/>
       <c r="B75" s="27" t="s">
         <v>301</v>
@@ -6727,7 +6733,7 @@
       <c r="F75" s="2"/>
       <c r="G75" s="2"/>
     </row>
-    <row r="76" ht="27" hidden="1" spans="1:7">
+    <row r="76" ht="27" spans="1:7">
       <c r="A76" s="2"/>
       <c r="B76" s="27" t="s">
         <v>303</v>
@@ -6744,9 +6750,9 @@
       <c r="F76" s="2"/>
       <c r="G76" s="2"/>
     </row>
-    <row r="77" ht="19.5" hidden="1" spans="1:7">
+    <row r="77" ht="19.5" spans="1:7">
       <c r="A77" s="2"/>
-      <c r="B77" s="36" t="s">
+      <c r="B77" s="37" t="s">
         <v>305</v>
       </c>
       <c r="C77" s="2"/>
@@ -6757,7 +6763,7 @@
       <c r="F77" s="2"/>
       <c r="G77" s="2"/>
     </row>
-    <row r="78" ht="16.5" hidden="1" spans="1:7">
+    <row r="78" ht="16.5" spans="1:7">
       <c r="A78" s="2"/>
       <c r="B78" s="2"/>
       <c r="C78" s="2"/>
@@ -6768,9 +6774,9 @@
       <c r="F78" s="2"/>
       <c r="G78" s="2"/>
     </row>
-    <row r="79" ht="19.5" hidden="1" spans="1:7">
+    <row r="79" ht="19.5" spans="1:7">
       <c r="A79" s="2"/>
-      <c r="B79" s="36" t="s">
+      <c r="B79" s="37" t="s">
         <v>306</v>
       </c>
       <c r="C79" s="2"/>
@@ -6781,7 +6787,7 @@
       <c r="F79" s="2"/>
       <c r="G79" s="2"/>
     </row>
-    <row r="80" ht="67.5" hidden="1" spans="1:7">
+    <row r="80" ht="67.5" spans="1:7">
       <c r="A80" s="2"/>
       <c r="B80" s="26" t="s">
         <v>307</v>
@@ -6798,7 +6804,7 @@
       <c r="F80" s="2"/>
       <c r="G80" s="2"/>
     </row>
-    <row r="81" ht="16.5" hidden="1" spans="1:7">
+    <row r="81" ht="16.5" spans="1:7">
       <c r="A81" s="2"/>
       <c r="B81" s="27" t="s">
         <v>309</v>
@@ -6813,11 +6819,11 @@
       <c r="F81" s="2"/>
       <c r="G81" s="2"/>
     </row>
-    <row r="82" ht="27" hidden="1" spans="1:7">
+    <row r="82" ht="27" spans="1:7">
       <c r="A82" s="2" t="s">
         <v>311</v>
       </c>
-      <c r="B82" s="37" t="s">
+      <c r="B82" s="38" t="s">
         <v>312</v>
       </c>
       <c r="C82" s="27" t="s">
@@ -6829,12 +6835,12 @@
       <c r="E82" s="27" t="s">
         <v>79</v>
       </c>
-      <c r="F82" s="2" t="s">
+      <c r="F82" s="30" t="s">
         <v>80</v>
       </c>
       <c r="G82" s="2"/>
     </row>
-    <row r="83" ht="16.5" hidden="1" spans="1:7">
+    <row r="83" ht="16.5" spans="1:7">
       <c r="A83" s="2"/>
       <c r="B83" s="2" t="s">
         <v>315</v>
@@ -6851,7 +6857,7 @@
       <c r="F83" s="2"/>
       <c r="G83" s="2"/>
     </row>
-    <row r="84" ht="27" hidden="1" spans="1:7">
+    <row r="84" ht="27" spans="1:7">
       <c r="A84" s="2"/>
       <c r="B84" s="2" t="s">
         <v>317</v>
@@ -6866,11 +6872,11 @@
       <c r="F84" s="2"/>
       <c r="G84" s="2"/>
     </row>
-    <row r="85" ht="16.5" hidden="1" spans="1:7">
-      <c r="A85" s="38" t="s">
+    <row r="85" ht="16.5" spans="1:7">
+      <c r="A85" s="39" t="s">
         <v>319</v>
       </c>
-      <c r="B85" s="39" t="s">
+      <c r="B85" s="40" t="s">
         <v>320</v>
       </c>
       <c r="C85" s="2"/>
@@ -6880,16 +6886,16 @@
       <c r="E85" s="27" t="s">
         <v>79</v>
       </c>
-      <c r="F85" s="2" t="s">
+      <c r="F85" s="30" t="s">
         <v>80</v>
       </c>
       <c r="G85" s="2"/>
     </row>
-    <row r="86" ht="54" hidden="1" spans="1:7">
-      <c r="A86" s="38" t="s">
+    <row r="86" ht="54" spans="1:7">
+      <c r="A86" s="39" t="s">
         <v>322</v>
       </c>
-      <c r="B86" s="39" t="s">
+      <c r="B86" s="40" t="s">
         <v>323</v>
       </c>
       <c r="C86" s="2" t="s">
@@ -6901,16 +6907,16 @@
       <c r="E86" s="27" t="s">
         <v>79</v>
       </c>
-      <c r="F86" s="2" t="s">
+      <c r="F86" s="30" t="s">
         <v>80</v>
       </c>
       <c r="G86" s="2"/>
     </row>
-    <row r="87" ht="16.5" hidden="1" spans="1:7">
+    <row r="87" ht="16.5" spans="1:7">
       <c r="A87" s="2" t="s">
         <v>325</v>
       </c>
-      <c r="B87" s="39" t="s">
+      <c r="B87" s="40" t="s">
         <v>326</v>
       </c>
       <c r="C87" s="2" t="s">
@@ -6922,12 +6928,12 @@
       <c r="E87" s="27" t="s">
         <v>79</v>
       </c>
-      <c r="F87" s="2" t="s">
+      <c r="F87" s="30" t="s">
         <v>80</v>
       </c>
       <c r="G87" s="2"/>
     </row>
-    <row r="88" ht="54" hidden="1" spans="1:7">
+    <row r="88" ht="54" spans="1:7">
       <c r="A88" s="2" t="s">
         <v>329</v>
       </c>
@@ -6948,7 +6954,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="89" ht="54" hidden="1" spans="1:7">
+    <row r="89" ht="54" spans="1:7">
       <c r="A89" s="2"/>
       <c r="B89" s="2" t="s">
         <v>333</v>
@@ -6963,7 +6969,7 @@
       <c r="F89" s="2"/>
       <c r="G89" s="2"/>
     </row>
-    <row r="90" ht="81" hidden="1" spans="1:7">
+    <row r="90" ht="81" spans="1:7">
       <c r="A90" s="2"/>
       <c r="B90" s="26" t="s">
         <v>335</v>
@@ -6978,11 +6984,11 @@
       <c r="F90" s="2"/>
       <c r="G90" s="2"/>
     </row>
-    <row r="91" ht="16.5" hidden="1" spans="1:7">
+    <row r="91" ht="16.5" spans="1:7">
       <c r="A91" s="2" t="s">
         <v>337</v>
       </c>
-      <c r="B91" s="40" t="s">
+      <c r="B91" s="30" t="s">
         <v>338</v>
       </c>
       <c r="C91" s="2" t="s">
@@ -6994,12 +7000,12 @@
       <c r="E91" s="27" t="s">
         <v>79</v>
       </c>
-      <c r="F91" s="2" t="s">
+      <c r="F91" s="30" t="s">
         <v>80</v>
       </c>
       <c r="G91" s="2"/>
     </row>
-    <row r="92" ht="27" hidden="1" spans="1:7">
+    <row r="92" ht="27" spans="1:7">
       <c r="A92" s="2"/>
       <c r="B92" s="2" t="s">
         <v>340</v>
@@ -7014,7 +7020,7 @@
       <c r="F92" s="2"/>
       <c r="G92" s="2"/>
     </row>
-    <row r="93" ht="30" hidden="1" spans="1:7">
+    <row r="93" ht="30" spans="1:7">
       <c r="A93" s="2" t="s">
         <v>342</v>
       </c>
@@ -7035,11 +7041,11 @@
         <v>21</v>
       </c>
     </row>
-    <row r="94" ht="81" hidden="1" spans="1:7">
+    <row r="94" ht="81" spans="1:7">
       <c r="A94" s="2" t="s">
         <v>345</v>
       </c>
-      <c r="B94" s="40" t="s">
+      <c r="B94" s="30" t="s">
         <v>346</v>
       </c>
       <c r="C94" s="2" t="s">
@@ -7051,12 +7057,12 @@
       <c r="E94" s="27" t="s">
         <v>79</v>
       </c>
-      <c r="F94" s="2" t="s">
+      <c r="F94" s="30" t="s">
         <v>80</v>
       </c>
       <c r="G94" s="2"/>
     </row>
-    <row r="95" ht="57" hidden="1" spans="1:7">
+    <row r="95" ht="57" spans="1:7">
       <c r="A95" s="2" t="s">
         <v>349</v>
       </c>
@@ -7077,11 +7083,11 @@
         <v>22</v>
       </c>
     </row>
-    <row r="96" customFormat="1" ht="27" hidden="1" spans="1:7">
+    <row r="96" customFormat="1" ht="27" spans="1:7">
       <c r="A96" s="2" t="s">
         <v>353</v>
       </c>
-      <c r="B96" s="40" t="s">
+      <c r="B96" s="30" t="s">
         <v>354</v>
       </c>
       <c r="C96" s="2" t="s">
@@ -7093,12 +7099,12 @@
       <c r="E96" s="2" t="s">
         <v>79</v>
       </c>
-      <c r="F96" s="2" t="s">
+      <c r="F96" s="30" t="s">
         <v>80</v>
       </c>
       <c r="G96" s="2"/>
     </row>
-    <row r="97" customFormat="1" ht="40.5" hidden="1" spans="1:7">
+    <row r="97" customFormat="1" ht="40.5" spans="1:7">
       <c r="A97" s="2"/>
       <c r="B97" s="2" t="s">
         <v>356</v>
@@ -7115,7 +7121,7 @@
       <c r="F97" s="2"/>
       <c r="G97" s="2"/>
     </row>
-    <row r="98" customFormat="1" hidden="1" spans="1:7">
+    <row r="98" customFormat="1" spans="1:7">
       <c r="A98" s="2"/>
       <c r="B98" s="2" t="s">
         <v>358</v>
@@ -7132,7 +7138,7 @@
       <c r="F98" s="2"/>
       <c r="G98" s="2"/>
     </row>
-    <row r="99" customFormat="1" ht="40.5" hidden="1" spans="1:7">
+    <row r="99" customFormat="1" ht="40.5" spans="1:7">
       <c r="A99" s="2" t="s">
         <v>361</v>
       </c>
@@ -7153,7 +7159,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="100" customFormat="1" ht="67.5" hidden="1" spans="1:7">
+    <row r="100" customFormat="1" ht="67.5" spans="1:7">
       <c r="A100" s="41" t="s">
         <v>364</v>
       </c>
@@ -7167,16 +7173,16 @@
       <c r="E100" s="2" t="s">
         <v>79</v>
       </c>
-      <c r="F100" s="2" t="s">
+      <c r="F100" s="30" t="s">
         <v>80</v>
       </c>
       <c r="G100" s="2"/>
     </row>
-    <row r="101" customFormat="1" ht="54" hidden="1" spans="1:7">
+    <row r="101" customFormat="1" ht="54" spans="1:7">
       <c r="A101" s="41" t="s">
         <v>367</v>
       </c>
-      <c r="B101" s="40" t="s">
+      <c r="B101" s="30" t="s">
         <v>368</v>
       </c>
       <c r="C101" s="2"/>
@@ -7186,12 +7192,12 @@
       <c r="E101" s="2" t="s">
         <v>79</v>
       </c>
-      <c r="F101" s="2" t="s">
+      <c r="F101" s="30" t="s">
         <v>80</v>
       </c>
       <c r="G101" s="2"/>
     </row>
-    <row r="102" customFormat="1" ht="67.5" hidden="1" spans="1:7">
+    <row r="102" customFormat="1" ht="67.5" spans="1:7">
       <c r="A102" s="2" t="s">
         <v>370</v>
       </c>
@@ -7212,7 +7218,7 @@
       </c>
       <c r="G102" s="2"/>
     </row>
-    <row r="103" customFormat="1" ht="54" hidden="1" spans="1:7">
+    <row r="103" customFormat="1" ht="54" spans="1:7">
       <c r="A103" s="2" t="s">
         <v>375</v>
       </c>
@@ -7233,11 +7239,11 @@
       </c>
       <c r="G103" s="2"/>
     </row>
-    <row r="104" customFormat="1" ht="54" hidden="1" spans="1:7">
+    <row r="104" customFormat="1" ht="54" spans="1:7">
       <c r="A104" s="2" t="s">
         <v>379</v>
       </c>
-      <c r="B104" s="40" t="s">
+      <c r="B104" s="30" t="s">
         <v>380</v>
       </c>
       <c r="C104" s="2" t="s">
@@ -7249,12 +7255,12 @@
       <c r="E104" s="2" t="s">
         <v>79</v>
       </c>
-      <c r="F104" s="2" t="s">
+      <c r="F104" s="30" t="s">
         <v>80</v>
       </c>
       <c r="G104" s="2"/>
     </row>
-    <row r="105" customFormat="1" ht="40.5" hidden="1" spans="1:7">
+    <row r="105" customFormat="1" ht="40.5" spans="1:7">
       <c r="A105" s="2" t="s">
         <v>383</v>
       </c>
@@ -7306,17 +7312,6 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" ref="A3:G105" etc:filterBottomFollowUsedRange="0">
-    <filterColumn colId="4">
-      <filters>
-        <filter val="P0"/>
-      </filters>
-    </filterColumn>
-    <filterColumn colId="5">
-      <filters blank="1"/>
-    </filterColumn>
-    <extLst/>
-  </autoFilter>
   <mergeCells count="2">
     <mergeCell ref="B1:E1"/>
     <mergeCell ref="B2:E2"/>

</xml_diff>